<commit_message>
pandas & spark update
</commit_message>
<xml_diff>
--- a/p/py-25/py-libs/pandas/topic-list_pandas.xlsx
+++ b/p/py-25/py-libs/pandas/topic-list_pandas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="17600" tabRatio="698" firstSheet="1"/>
+    <workbookView windowHeight="17600" tabRatio="698" firstSheet="1"/>
   </bookViews>
   <sheets>
     <sheet name="what" sheetId="21" r:id="rId1"/>
@@ -12,12 +12,7 @@
     <sheet name="ex" sheetId="17" r:id="rId3"/>
     <sheet name="casting" sheetId="3" r:id="rId4"/>
     <sheet name="intermed" sheetId="5" r:id="rId5"/>
-    <sheet name="adv" sheetId="15" r:id="rId6"/>
-    <sheet name="module" sheetId="9" r:id="rId7"/>
-    <sheet name="ques" sheetId="6" r:id="rId8"/>
-    <sheet name="-" sheetId="8" r:id="rId9"/>
-    <sheet name="other topics" sheetId="12" r:id="rId10"/>
-    <sheet name="ex libs" sheetId="20" r:id="rId11"/>
+    <sheet name="ques" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="271">
   <si>
     <t>Data Wrangling with pandas Cheat Sheet</t>
   </si>
@@ -958,12 +953,6 @@
     </r>
   </si>
   <si>
-    <t>Advance and less used things in py</t>
-  </si>
-  <si>
-    <t>Common modules which can be used anywhere</t>
-  </si>
-  <si>
     <t>duplicate index/col detect</t>
   </si>
   <si>
@@ -1035,7 +1024,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="28">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1050,39 +1039,14 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF282829"/>
-      <name val="Bahnschrift"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF282829"/>
-      <name val="Bahnschrift"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF040C28"/>
-      <name val="Bahnschrift"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Bahnschrift"/>
+      <sz val="10.5"/>
+      <color rgb="FF080808"/>
+      <name val="Consolas"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Bahnschrift"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10.5"/>
-      <color rgb="FF080808"/>
-      <name val="Consolas"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1251,13 +1215,13 @@
     </font>
     <font>
       <sz val="10.5"/>
-      <color rgb="FF222832"/>
+      <color rgb="FF00622F"/>
       <name val="Consolas"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="10.5"/>
-      <color rgb="FF00622F"/>
+      <color rgb="FF222832"/>
       <name val="Consolas"/>
       <charset val="134"/>
     </font>
@@ -1595,213 +1559,189 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -2175,7 +2115,7 @@
       </c>
     </row>
     <row r="7" spans="2:2">
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="23" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2201,429 +2141,6 @@
       <c r="A12">
         <v>3</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A8:D42"/>
-  <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5" outlineLevelCol="3"/>
-  <cols>
-    <col min="1" max="1" width="8.66923076923077" style="8"/>
-    <col min="2" max="2" width="14.6923076923077" style="8" customWidth="1"/>
-    <col min="3" max="3" width="22.3846153846154" style="8" customWidth="1"/>
-    <col min="4" max="16384" width="8.66923076923077" style="8"/>
-  </cols>
-  <sheetData>
-    <row r="8" ht="14" spans="4:4">
-      <c r="D8" s="9"/>
-    </row>
-    <row r="13" ht="14" spans="1:4">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-    </row>
-    <row r="14" ht="14" spans="1:4">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-    </row>
-    <row r="15" ht="14" spans="1:4">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-    </row>
-    <row r="16" ht="14" spans="1:4">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-    </row>
-    <row r="17" ht="14" spans="1:4">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-    </row>
-    <row r="18" ht="14" spans="1:4">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-    </row>
-    <row r="19" ht="14" spans="1:4">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-    </row>
-    <row r="20" ht="14" spans="1:4">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-    </row>
-    <row r="21" ht="14" spans="1:4">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-    </row>
-    <row r="22" ht="14" spans="1:4">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-    </row>
-    <row r="23" ht="14" spans="1:4">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-    </row>
-    <row r="24" ht="14" spans="1:4">
-      <c r="A24" s="10"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-    </row>
-    <row r="25" ht="14" spans="1:4">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-    </row>
-    <row r="26" ht="14" spans="1:4">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-    </row>
-    <row r="27" ht="14" spans="1:4">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-    </row>
-    <row r="28" ht="14" spans="1:4">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-    </row>
-    <row r="29" ht="14" spans="1:4">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-    </row>
-    <row r="30" ht="14" spans="1:4">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-    </row>
-    <row r="31" ht="14" spans="1:4">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-    </row>
-    <row r="32" ht="14" spans="1:4">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-    </row>
-    <row r="33" ht="14" spans="1:4">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-    </row>
-    <row r="34" ht="14" spans="1:4">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-    </row>
-    <row r="35" ht="14" spans="1:4">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-    </row>
-    <row r="36" ht="14" spans="1:4">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-    </row>
-    <row r="37" ht="14" spans="1:4">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-    </row>
-    <row r="38" ht="14" spans="1:4">
-      <c r="A38" s="10"/>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-    </row>
-    <row r="39" ht="14" spans="1:4">
-      <c r="A39" s="10"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-    </row>
-    <row r="40" ht="14" spans="1:4">
-      <c r="A40" s="10"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-    </row>
-    <row r="41" ht="14" spans="1:4">
-      <c r="A41" s="10"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-    </row>
-    <row r="42" ht="14" spans="1:4">
-      <c r="A42" s="10"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A2:A73"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="14"/>
-  <cols>
-    <col min="1" max="16384" width="9.23076923076923" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:1">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="3"/>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="4"/>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="3"/>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="5"/>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="5"/>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="6"/>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" s="6"/>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" s="6"/>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" s="5"/>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" s="3"/>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" s="4"/>
-    </row>
-    <row r="14" spans="1:1">
-      <c r="A14" s="3"/>
-    </row>
-    <row r="15" spans="1:1">
-      <c r="A15" s="5"/>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" s="5"/>
-    </row>
-    <row r="17" spans="1:1">
-      <c r="A17" s="6"/>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" s="6"/>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" s="6"/>
-    </row>
-    <row r="20" spans="1:1">
-      <c r="A20" s="5"/>
-    </row>
-    <row r="21" spans="1:1">
-      <c r="A21" s="3"/>
-    </row>
-    <row r="22" spans="1:1">
-      <c r="A22" s="4"/>
-    </row>
-    <row r="23" spans="1:1">
-      <c r="A23" s="3"/>
-    </row>
-    <row r="24" spans="1:1">
-      <c r="A24" s="3"/>
-    </row>
-    <row r="25" spans="1:1">
-      <c r="A25" s="5"/>
-    </row>
-    <row r="26" spans="1:1">
-      <c r="A26" s="5"/>
-    </row>
-    <row r="27" spans="1:1">
-      <c r="A27" s="6"/>
-    </row>
-    <row r="28" spans="1:1">
-      <c r="A28" s="6"/>
-    </row>
-    <row r="29" spans="1:1">
-      <c r="A29" s="6"/>
-    </row>
-    <row r="30" spans="1:1">
-      <c r="A30" s="5"/>
-    </row>
-    <row r="31" spans="1:1">
-      <c r="A31" s="3"/>
-    </row>
-    <row r="32" spans="1:1">
-      <c r="A32" s="4"/>
-    </row>
-    <row r="33" spans="1:1">
-      <c r="A33" s="3"/>
-    </row>
-    <row r="34" spans="1:1">
-      <c r="A34" s="5"/>
-    </row>
-    <row r="35" spans="1:1">
-      <c r="A35" s="5"/>
-    </row>
-    <row r="36" spans="1:1">
-      <c r="A36" s="6"/>
-    </row>
-    <row r="37" spans="1:1">
-      <c r="A37" s="6"/>
-    </row>
-    <row r="38" spans="1:1">
-      <c r="A38" s="6"/>
-    </row>
-    <row r="39" spans="1:1">
-      <c r="A39" s="5"/>
-    </row>
-    <row r="40" spans="1:1">
-      <c r="A40" s="3"/>
-    </row>
-    <row r="41" spans="1:1">
-      <c r="A41" s="4"/>
-    </row>
-    <row r="42" spans="1:1">
-      <c r="A42" s="3"/>
-    </row>
-    <row r="43" spans="1:1">
-      <c r="A43" s="5"/>
-    </row>
-    <row r="44" spans="1:1">
-      <c r="A44" s="5"/>
-    </row>
-    <row r="45" spans="1:1">
-      <c r="A45" s="6"/>
-    </row>
-    <row r="46" spans="1:1">
-      <c r="A46" s="6"/>
-    </row>
-    <row r="47" spans="1:1">
-      <c r="A47" s="6"/>
-    </row>
-    <row r="48" spans="1:1">
-      <c r="A48" s="5"/>
-    </row>
-    <row r="49" spans="1:1">
-      <c r="A49" s="3"/>
-    </row>
-    <row r="50" spans="1:1">
-      <c r="A50" s="4"/>
-    </row>
-    <row r="51" spans="1:1">
-      <c r="A51" s="3"/>
-    </row>
-    <row r="52" spans="1:1">
-      <c r="A52" s="5"/>
-    </row>
-    <row r="53" spans="1:1">
-      <c r="A53" s="5"/>
-    </row>
-    <row r="54" spans="1:1">
-      <c r="A54" s="6"/>
-    </row>
-    <row r="55" spans="1:1">
-      <c r="A55" s="6"/>
-    </row>
-    <row r="56" spans="1:1">
-      <c r="A56" s="6"/>
-    </row>
-    <row r="57" spans="1:1">
-      <c r="A57" s="5"/>
-    </row>
-    <row r="58" spans="1:1">
-      <c r="A58" s="3"/>
-    </row>
-    <row r="59" spans="1:1">
-      <c r="A59" s="4"/>
-    </row>
-    <row r="60" spans="1:1">
-      <c r="A60" s="3"/>
-    </row>
-    <row r="61" spans="1:1">
-      <c r="A61" s="5"/>
-    </row>
-    <row r="62" spans="1:1">
-      <c r="A62" s="5"/>
-    </row>
-    <row r="63" spans="1:1">
-      <c r="A63" s="6"/>
-    </row>
-    <row r="64" spans="1:1">
-      <c r="A64" s="6"/>
-    </row>
-    <row r="65" spans="1:1">
-      <c r="A65" s="6"/>
-    </row>
-    <row r="66" spans="1:1">
-      <c r="A66" s="5"/>
-    </row>
-    <row r="67" spans="1:1">
-      <c r="A67" s="3"/>
-    </row>
-    <row r="68" spans="1:1">
-      <c r="A68" s="4"/>
-    </row>
-    <row r="69" spans="1:1">
-      <c r="A69" s="2"/>
-    </row>
-    <row r="73" spans="1:1">
-      <c r="A73" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2637,628 +2154,628 @@
   <dimension ref="A1:H93"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="27.3307692307692" style="26" customWidth="1"/>
-    <col min="2" max="2" width="19.8307692307692" style="26" customWidth="1"/>
-    <col min="3" max="3" width="2.41538461538462" style="26" customWidth="1"/>
-    <col min="4" max="4" width="3.33076923076923" style="26" customWidth="1"/>
-    <col min="5" max="5" width="12.6692307692308" style="26" customWidth="1"/>
-    <col min="6" max="6" width="12.1692307692308" style="26" customWidth="1"/>
-    <col min="7" max="8" width="4.5" style="26" customWidth="1"/>
-    <col min="9" max="16384" width="11" style="26"/>
+    <col min="1" max="1" width="27.3307692307692" style="16" customWidth="1"/>
+    <col min="2" max="2" width="19.8307692307692" style="16" customWidth="1"/>
+    <col min="3" max="3" width="2.41538461538462" style="16" customWidth="1"/>
+    <col min="4" max="4" width="3.33076923076923" style="16" customWidth="1"/>
+    <col min="5" max="5" width="12.6692307692308" style="16" customWidth="1"/>
+    <col min="6" max="6" width="12.1692307692308" style="16" customWidth="1"/>
+    <col min="7" max="8" width="4.5" style="16" customWidth="1"/>
+    <col min="9" max="16384" width="11" style="16"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="16" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="27" t="s">
+      <c r="G2" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="26" t="s">
+      <c r="H2" s="16" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="3:3">
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="4:4">
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="16" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="16" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6" spans="4:4">
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="16" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="4:4">
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="16" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="2:6">
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="16" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" ht="56" spans="1:5">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="16" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="16" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="16" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="4:4">
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="16" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="26" t="s">
+      <c r="E13" s="16" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="4:4">
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="5:5">
-      <c r="E15" s="26" t="s">
+      <c r="E15" s="16" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="16" spans="2:5">
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="16" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="17" spans="5:5">
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="16" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="18" spans="4:4">
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="16" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="19" spans="4:4">
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="16" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="20" spans="4:4">
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="16" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="23" spans="4:4">
-      <c r="D23" s="26" t="s">
+      <c r="D23" s="16" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="24" spans="4:4">
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="16" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="25" spans="5:5">
-      <c r="E25" s="26" t="s">
+      <c r="E25" s="16" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="26" spans="5:5">
-      <c r="E26" s="26" t="s">
+      <c r="E26" s="16" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="26" t="s">
+      <c r="A27" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="26" t="s">
+      <c r="E27" s="16" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="28" spans="4:4">
-      <c r="D28" s="26" t="s">
+      <c r="D28" s="16" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="29" spans="5:5">
-      <c r="E29" s="26" t="s">
+      <c r="E29" s="16" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="30"/>
-      <c r="B30" s="30"/>
-      <c r="E30" s="26" t="s">
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
+      <c r="E30" s="16" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="30"/>
-      <c r="B31" s="30"/>
-      <c r="E31" s="26" t="s">
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
+      <c r="E31" s="16" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:5">
-      <c r="A32" s="30"/>
-      <c r="B32" s="30"/>
-      <c r="E32" s="26" t="s">
+      <c r="A32" s="20"/>
+      <c r="B32" s="20"/>
+      <c r="E32" s="16" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="30"/>
-      <c r="B33" s="26" t="s">
+      <c r="A33" s="20"/>
+      <c r="B33" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="E33" s="26" t="s">
+      <c r="E33" s="16" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="30"/>
-      <c r="B34" s="30"/>
-      <c r="E34" s="26" t="s">
+      <c r="A34" s="20"/>
+      <c r="B34" s="20"/>
+      <c r="E34" s="16" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="26" t="s">
+      <c r="A35" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B35" s="26" t="s">
+      <c r="B35" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="E35" s="26" t="s">
+      <c r="E35" s="16" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="36" spans="2:5">
-      <c r="B36" s="26" t="s">
+      <c r="B36" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="E36" s="26" t="s">
+      <c r="E36" s="16" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="37" spans="5:5">
-      <c r="E37" s="26" t="s">
+      <c r="E37" s="16" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="38" spans="1:5">
-      <c r="A38" s="26" t="s">
+      <c r="A38" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B38" s="26" t="s">
+      <c r="B38" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="E38" s="26" t="s">
+      <c r="E38" s="16" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="30"/>
-      <c r="D39" s="26" t="s">
+      <c r="A39" s="20"/>
+      <c r="D39" s="16" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="40" spans="1:5">
-      <c r="A40" s="30"/>
-      <c r="B40" s="26" t="s">
+      <c r="A40" s="20"/>
+      <c r="B40" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="E40" s="26" t="s">
+      <c r="E40" s="16" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" s="30"/>
-      <c r="D41" s="26" t="s">
+      <c r="A41" s="20"/>
+      <c r="D41" s="16" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="42" spans="2:5">
-      <c r="B42" s="26" t="s">
+      <c r="B42" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="E42" s="26" t="s">
+      <c r="E42" s="16" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" s="30"/>
-      <c r="D43" s="26" t="s">
+      <c r="A43" s="20"/>
+      <c r="D43" s="16" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="44" spans="2:5">
-      <c r="B44" s="26" t="s">
+      <c r="B44" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="E44" s="26" t="s">
+      <c r="E44" s="16" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="45" spans="2:2">
-      <c r="B45" s="26" t="s">
+      <c r="B45" s="16" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="47" spans="4:4">
-      <c r="D47" s="26" t="s">
+      <c r="D47" s="16" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="26" t="s">
+      <c r="A48" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B48" s="26" t="s">
+      <c r="B48" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="E48" s="26" t="s">
+      <c r="E48" s="16" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="49" spans="1:2">
-      <c r="A49" s="26" t="s">
+      <c r="A49" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="B49" s="26" t="s">
+      <c r="B49" s="16" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="50" spans="2:2">
-      <c r="B50" s="26" t="s">
+      <c r="B50" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="26" t="s">
+      <c r="A51" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="E51" s="26" t="s">
+      <c r="E51" s="16" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="52" spans="2:6">
-      <c r="B52" s="26" t="s">
+      <c r="B52" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="F52" s="26" t="s">
+      <c r="F52" s="16" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="53" spans="2:4">
-      <c r="B53" s="26" t="s">
+      <c r="B53" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="D53" s="26" t="s">
+      <c r="D53" s="16" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="54" spans="2:2">
-      <c r="B54" s="26" t="s">
+      <c r="B54" s="16" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="55" spans="5:5">
-      <c r="E55" s="26" t="s">
+      <c r="E55" s="16" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="56" spans="1:4">
-      <c r="A56" s="26" t="s">
+      <c r="A56" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B56" s="26" t="s">
+      <c r="B56" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="D56" s="31" t="s">
+      <c r="D56" s="21" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="57" spans="1:4">
-      <c r="A57" s="26" t="s">
+      <c r="A57" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B57" s="26" t="s">
+      <c r="B57" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="D57" s="31" t="s">
+      <c r="D57" s="21" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="58" spans="4:4">
-      <c r="D58" s="20" t="s">
+      <c r="D58" s="8" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="60" spans="4:4">
-      <c r="D60" s="26" t="s">
+      <c r="D60" s="16" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="61" spans="1:6">
-      <c r="A61" s="26" t="s">
+      <c r="A61" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B61" s="26" t="s">
+      <c r="B61" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="C61" s="30"/>
-      <c r="D61" s="30"/>
-      <c r="E61" s="30"/>
-      <c r="F61" s="30" t="s">
+      <c r="C61" s="20"/>
+      <c r="D61" s="20"/>
+      <c r="E61" s="20"/>
+      <c r="F61" s="20" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="62" spans="2:6">
-      <c r="B62" s="26" t="s">
+      <c r="B62" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="C62" s="30"/>
-      <c r="D62" s="30"/>
-      <c r="E62" s="30"/>
-      <c r="F62" s="30"/>
+      <c r="C62" s="20"/>
+      <c r="D62" s="20"/>
+      <c r="E62" s="20"/>
+      <c r="F62" s="20"/>
     </row>
     <row r="63" spans="3:6">
-      <c r="C63" s="30"/>
-      <c r="D63" s="30"/>
-      <c r="E63" s="30"/>
-      <c r="F63" s="30"/>
+      <c r="C63" s="20"/>
+      <c r="D63" s="20"/>
+      <c r="E63" s="20"/>
+      <c r="F63" s="20"/>
     </row>
     <row r="64" spans="2:6">
-      <c r="B64" s="26" t="s">
+      <c r="B64" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="C64" s="30"/>
-      <c r="D64" s="30"/>
-      <c r="E64" s="26" t="s">
+      <c r="C64" s="20"/>
+      <c r="D64" s="20"/>
+      <c r="E64" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="F64" s="30"/>
+      <c r="F64" s="20"/>
     </row>
     <row r="65" spans="2:6">
-      <c r="B65" s="26" t="s">
+      <c r="B65" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="C65" s="30"/>
-      <c r="D65" s="30"/>
-      <c r="E65" s="30"/>
-      <c r="F65" s="30"/>
+      <c r="C65" s="20"/>
+      <c r="D65" s="20"/>
+      <c r="E65" s="20"/>
+      <c r="F65" s="20"/>
     </row>
     <row r="66" spans="3:6">
-      <c r="C66" s="30"/>
-      <c r="D66" s="30"/>
-      <c r="E66" s="30"/>
-      <c r="F66" s="30"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
     </row>
     <row r="67" spans="3:3">
-      <c r="C67" s="26" t="s">
+      <c r="C67" s="16" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="68" spans="4:4">
-      <c r="D68" s="26" t="s">
+      <c r="D68" s="16" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="69" spans="4:4">
-      <c r="D69" s="26" t="s">
+      <c r="D69" s="16" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="70" spans="4:4">
-      <c r="D70" s="26" t="s">
+      <c r="D70" s="16" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="71" spans="1:4">
-      <c r="A71" s="26" t="s">
+      <c r="A71" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B71" s="26" t="s">
+      <c r="B71" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="D71" s="26" t="s">
+      <c r="D71" s="16" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="72" spans="3:3">
-      <c r="C72" s="26" t="s">
+      <c r="C72" s="16" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="73" spans="4:4">
-      <c r="D73" s="26" t="s">
+      <c r="D73" s="16" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="74" spans="1:4">
-      <c r="A74" s="26" t="s">
+      <c r="A74" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B74" s="26" t="s">
+      <c r="B74" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="D74" s="26" t="s">
+      <c r="D74" s="16" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="75" spans="3:3">
-      <c r="C75" s="26" t="s">
+      <c r="C75" s="16" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="76" spans="4:4">
-      <c r="D76" s="26" t="s">
+      <c r="D76" s="16" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="77" spans="4:4">
-      <c r="D77" s="26" t="s">
+      <c r="D77" s="16" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="78" spans="1:4">
-      <c r="A78" s="26" t="s">
+      <c r="A78" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B78" s="26" t="s">
+      <c r="B78" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="D78" s="26" t="s">
+      <c r="D78" s="16" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="79" spans="2:2">
-      <c r="B79" s="26" t="s">
+      <c r="B79" s="16" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="80" spans="2:2">
-      <c r="B80" s="32" t="s">
+      <c r="B80" s="22" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="81" spans="1:2">
-      <c r="A81" s="26" t="s">
+      <c r="A81" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="B81" s="32" t="s">
+      <c r="B81" s="22" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="82" spans="2:4">
-      <c r="B82" s="32"/>
-      <c r="D82" s="26" t="s">
+      <c r="B82" s="22"/>
+      <c r="D82" s="16" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="83" spans="1:2">
-      <c r="A83" s="26" t="s">
+      <c r="A83" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="B83" s="32" t="s">
+      <c r="B83" s="22" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="84" spans="2:2">
-      <c r="B84" s="32"/>
+      <c r="B84" s="22"/>
     </row>
     <row r="85" spans="3:3">
-      <c r="C85" s="26" t="s">
+      <c r="C85" s="16" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="86" spans="1:4">
-      <c r="A86" s="26" t="s">
+      <c r="A86" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="B86" s="26" t="s">
+      <c r="B86" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="D86" s="26" t="s">
+      <c r="D86" s="16" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="87" spans="2:5">
-      <c r="B87" s="26" t="s">
+      <c r="B87" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="E87" s="26" t="s">
+      <c r="E87" s="16" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="88" spans="4:4">
-      <c r="D88" s="31" t="s">
+      <c r="D88" s="21" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="90" spans="3:3">
-      <c r="C90" s="26" t="s">
+      <c r="C90" s="16" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="91" spans="4:4">
-      <c r="D91" s="26" t="s">
+      <c r="D91" s="16" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="92" spans="3:3">
-      <c r="C92" s="26" t="s">
+      <c r="C92" s="16" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="93" spans="4:4">
-      <c r="D93" s="26" t="s">
+      <c r="D93" s="16" t="s">
         <v>127</v>
       </c>
     </row>
@@ -3275,38 +2792,38 @@
   <dimension ref="A1:H95"/>
   <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="14" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="25.5" style="13" customWidth="1"/>
-    <col min="2" max="2" width="19.8307692307692" style="13" customWidth="1"/>
-    <col min="3" max="3" width="2.41538461538462" style="13" customWidth="1"/>
-    <col min="4" max="4" width="3.33076923076923" style="13" customWidth="1"/>
-    <col min="5" max="5" width="12.6692307692308" style="13" customWidth="1"/>
-    <col min="6" max="6" width="12.1692307692308" style="13" customWidth="1"/>
-    <col min="7" max="8" width="4.5" style="13" customWidth="1"/>
-    <col min="9" max="16384" width="8.66923076923077" style="13"/>
+    <col min="1" max="1" width="25.5" style="4" customWidth="1"/>
+    <col min="2" max="2" width="19.8307692307692" style="4" customWidth="1"/>
+    <col min="3" max="3" width="2.41538461538462" style="4" customWidth="1"/>
+    <col min="4" max="4" width="3.33076923076923" style="4" customWidth="1"/>
+    <col min="5" max="5" width="12.6692307692308" style="4" customWidth="1"/>
+    <col min="6" max="6" width="12.1692307692308" style="4" customWidth="1"/>
+    <col min="7" max="8" width="4.5" style="4" customWidth="1"/>
+    <col min="9" max="16384" width="8.66923076923077" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="4" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="4" t="s">
         <v>14</v>
       </c>
     </row>
@@ -3335,7 +2852,7 @@
       <c r="F5" s="10"/>
     </row>
     <row r="6" spans="2:6">
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="4" t="s">
         <v>132</v>
       </c>
       <c r="C6" s="10"/>
@@ -3356,7 +2873,7 @@
       </c>
     </row>
     <row r="8" spans="2:6">
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="11" t="s">
         <v>136</v>
       </c>
       <c r="C8" s="10"/>
@@ -3367,7 +2884,7 @@
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="4" t="s">
         <v>137</v>
       </c>
       <c r="F9" s="10"/>
@@ -3376,10 +2893,10 @@
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="4" t="s">
         <v>139</v>
       </c>
     </row>
@@ -3517,7 +3034,7 @@
       <c r="E28" s="10"/>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="4" t="s">
         <v>154</v>
       </c>
       <c r="C29" s="10"/>
@@ -3535,782 +3052,782 @@
       <c r="C31" s="10"/>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="4" t="s">
         <v>156</v>
       </c>
       <c r="C32" s="10"/>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="4" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:8">
-      <c r="A33" s="22"/>
-      <c r="B33" s="22"/>
-      <c r="C33" s="22" t="s">
+      <c r="A33" s="12"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="23"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="13"/>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:8">
-      <c r="A34" s="22"/>
-      <c r="B34" s="22" t="s">
+      <c r="A34" s="12"/>
+      <c r="B34" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22" t="s">
+      <c r="C34" s="12"/>
+      <c r="D34" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="23"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="13"/>
+      <c r="H34" s="13"/>
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:8">
-      <c r="A35" s="22"/>
-      <c r="B35" s="22" t="s">
+      <c r="A35" s="12"/>
+      <c r="B35" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22" t="s">
+      <c r="C35" s="12"/>
+      <c r="D35" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="23"/>
-      <c r="H35" s="23"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="13"/>
+      <c r="H35" s="13"/>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:8">
-      <c r="A36" s="22"/>
-      <c r="B36" s="22" t="s">
+      <c r="A36" s="12"/>
+      <c r="B36" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22" t="s">
+      <c r="C36" s="12"/>
+      <c r="D36" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="23"/>
-      <c r="H36" s="23"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="13"/>
+      <c r="H36" s="13"/>
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:8">
-      <c r="A37" s="22"/>
-      <c r="B37" s="22" t="s">
+      <c r="A37" s="12"/>
+      <c r="B37" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="C37" s="22"/>
-      <c r="D37" s="22" t="s">
+      <c r="C37" s="12"/>
+      <c r="D37" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="23"/>
-      <c r="H37" s="23"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="13"/>
+      <c r="H37" s="13"/>
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:8">
-      <c r="A38" s="22"/>
-      <c r="B38" s="22" t="s">
+      <c r="A38" s="12"/>
+      <c r="B38" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="C38" s="22"/>
-      <c r="D38" s="22" t="s">
+      <c r="C38" s="12"/>
+      <c r="D38" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="23"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="13"/>
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:8">
-      <c r="A39" s="22"/>
-      <c r="B39" s="22"/>
-      <c r="C39" s="22"/>
+      <c r="A39" s="12"/>
+      <c r="B39" s="12"/>
+      <c r="C39" s="12"/>
       <c r="D39" s="10"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="23"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="13"/>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:8">
-      <c r="A40" s="22"/>
-      <c r="B40" s="22"/>
-      <c r="C40" s="22"/>
+      <c r="A40" s="12"/>
+      <c r="B40" s="12"/>
+      <c r="C40" s="12"/>
       <c r="D40" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="23"/>
+      <c r="E40" s="12"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="13"/>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:8">
-      <c r="A41" s="22"/>
-      <c r="B41" s="22"/>
-      <c r="C41" s="22"/>
+      <c r="A41" s="12"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="12"/>
       <c r="D41" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="23"/>
+      <c r="E41" s="12"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="13"/>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:8">
-      <c r="A42" s="22" t="s">
+      <c r="A42" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="B42" s="22" t="s">
+      <c r="B42" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22" t="s">
+      <c r="C42" s="12"/>
+      <c r="D42" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="19"/>
-      <c r="H42" s="23"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="13"/>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:8">
-      <c r="A43" s="22"/>
-      <c r="B43" s="22"/>
-      <c r="C43" s="22"/>
-      <c r="D43" s="22"/>
-      <c r="E43" s="22" t="s">
+      <c r="A43" s="12"/>
+      <c r="B43" s="12"/>
+      <c r="C43" s="12"/>
+      <c r="D43" s="12"/>
+      <c r="E43" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="F43" s="22"/>
-      <c r="G43" s="19"/>
-      <c r="H43" s="23"/>
+      <c r="F43" s="12"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="13"/>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:8">
-      <c r="A44" s="22"/>
-      <c r="B44" s="22"/>
-      <c r="C44" s="22"/>
-      <c r="D44" s="22"/>
-      <c r="E44" s="22" t="s">
+      <c r="A44" s="12"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="F44" s="22"/>
-      <c r="G44" s="19"/>
-      <c r="H44" s="23"/>
+      <c r="F44" s="12"/>
+      <c r="G44" s="7"/>
+      <c r="H44" s="13"/>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:8">
-      <c r="A45" s="22"/>
-      <c r="B45" s="22"/>
-      <c r="C45" s="22"/>
-      <c r="D45" s="22"/>
-      <c r="E45" s="22" t="s">
+      <c r="A45" s="12"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="12"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="F45" s="22"/>
-      <c r="G45" s="19"/>
-      <c r="H45" s="23"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="13"/>
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:8">
-      <c r="A46" s="22"/>
-      <c r="B46" s="22"/>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22" t="s">
+      <c r="A46" s="12"/>
+      <c r="B46" s="12"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="F46" s="22"/>
-      <c r="G46" s="19"/>
-      <c r="H46" s="23"/>
+      <c r="F46" s="12"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="13"/>
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:8">
-      <c r="A47" s="22"/>
-      <c r="B47" s="22"/>
-      <c r="C47" s="22"/>
-      <c r="D47" s="22"/>
-      <c r="E47" s="22" t="s">
+      <c r="A47" s="12"/>
+      <c r="B47" s="12"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="F47" s="22"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="23"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="13"/>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:8">
-      <c r="A48" s="22"/>
-      <c r="B48" s="22" t="s">
+      <c r="A48" s="12"/>
+      <c r="B48" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22" t="s">
+      <c r="C48" s="12"/>
+      <c r="D48" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="19"/>
-      <c r="H48" s="23"/>
+      <c r="E48" s="12"/>
+      <c r="F48" s="12"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="13"/>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:8">
-      <c r="A49" s="22"/>
-      <c r="B49" s="22" t="s">
+      <c r="A49" s="12"/>
+      <c r="B49" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="C49" s="22"/>
-      <c r="D49" s="22" t="s">
+      <c r="C49" s="12"/>
+      <c r="D49" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="E49" s="22"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="19"/>
-      <c r="H49" s="23"/>
+      <c r="E49" s="12"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="13"/>
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:8">
-      <c r="A50" s="22"/>
-      <c r="B50" s="22" t="s">
+      <c r="A50" s="12"/>
+      <c r="B50" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="C50" s="22"/>
-      <c r="D50" s="22" t="s">
+      <c r="C50" s="12"/>
+      <c r="D50" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22"/>
-      <c r="G50" s="19"/>
-      <c r="H50" s="23"/>
+      <c r="E50" s="12"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="13"/>
     </row>
     <row r="51" ht="16" customHeight="1" spans="1:8">
-      <c r="A51" s="22"/>
-      <c r="B51" s="22" t="s">
+      <c r="A51" s="12"/>
+      <c r="B51" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="C51" s="22"/>
-      <c r="D51" s="22" t="s">
+      <c r="C51" s="12"/>
+      <c r="D51" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="E51" s="22"/>
-      <c r="F51" s="22"/>
-      <c r="G51" s="19"/>
-      <c r="H51" s="23"/>
+      <c r="E51" s="12"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="13"/>
     </row>
     <row r="52" ht="16" customHeight="1" spans="1:8">
-      <c r="A52" s="22"/>
-      <c r="B52" s="22"/>
-      <c r="C52" s="22"/>
-      <c r="D52" s="22"/>
-      <c r="E52" s="22" t="s">
+      <c r="A52" s="12"/>
+      <c r="B52" s="12"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="12"/>
+      <c r="E52" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="F52" s="22"/>
-      <c r="G52" s="19"/>
-      <c r="H52" s="23"/>
+      <c r="F52" s="12"/>
+      <c r="G52" s="7"/>
+      <c r="H52" s="13"/>
     </row>
     <row r="53" ht="16" customHeight="1" spans="1:8">
-      <c r="A53" s="22"/>
-      <c r="B53" s="22" t="s">
+      <c r="A53" s="12"/>
+      <c r="B53" s="12" t="s">
         <v>188</v>
       </c>
-      <c r="C53" s="22"/>
-      <c r="D53" s="22"/>
-      <c r="E53" s="22" t="s">
+      <c r="C53" s="12"/>
+      <c r="D53" s="12"/>
+      <c r="E53" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="F53" s="22"/>
-      <c r="G53" s="19"/>
-      <c r="H53" s="23"/>
+      <c r="F53" s="12"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="13"/>
     </row>
     <row r="54" ht="16" customHeight="1" spans="1:8">
-      <c r="A54" s="22"/>
-      <c r="B54" s="22" t="s">
+      <c r="A54" s="12"/>
+      <c r="B54" s="12" t="s">
         <v>190</v>
       </c>
-      <c r="C54" s="22"/>
-      <c r="D54" s="22"/>
-      <c r="E54" s="22" t="s">
+      <c r="C54" s="12"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="F54" s="22"/>
-      <c r="G54" s="19"/>
-      <c r="H54" s="23"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="13"/>
     </row>
     <row r="55" ht="16" customHeight="1" spans="1:8">
-      <c r="A55" s="22"/>
-      <c r="B55" s="22"/>
-      <c r="C55" s="22" t="s">
+      <c r="A55" s="12"/>
+      <c r="B55" s="12"/>
+      <c r="C55" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="D55" s="22"/>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="19"/>
-      <c r="H55" s="23"/>
+      <c r="D55" s="12"/>
+      <c r="E55" s="12"/>
+      <c r="F55" s="12"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="13"/>
     </row>
     <row r="56" ht="16" customHeight="1" spans="1:8">
-      <c r="A56" s="22"/>
-      <c r="B56" s="22"/>
-      <c r="C56" s="22"/>
-      <c r="D56" s="22" t="s">
+      <c r="A56" s="12"/>
+      <c r="B56" s="12"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="23"/>
+      <c r="E56" s="12"/>
+      <c r="F56" s="12"/>
+      <c r="G56" s="7"/>
+      <c r="H56" s="13"/>
     </row>
     <row r="57" ht="16" customHeight="1" spans="1:8">
-      <c r="A57" s="22"/>
-      <c r="B57" s="22" t="s">
+      <c r="A57" s="12"/>
+      <c r="B57" s="12" t="s">
         <v>194</v>
       </c>
-      <c r="C57" s="22"/>
-      <c r="D57" s="22"/>
-      <c r="E57" s="22" t="s">
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="F57" s="22"/>
-      <c r="G57" s="19"/>
-      <c r="H57" s="23"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="13"/>
     </row>
     <row r="58" ht="16" customHeight="1" spans="1:8">
-      <c r="A58" s="22"/>
-      <c r="B58" s="22"/>
-      <c r="C58" s="22"/>
-      <c r="D58" s="22"/>
-      <c r="E58" s="22" t="s">
+      <c r="A58" s="12"/>
+      <c r="B58" s="12"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="F58" s="22"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="23"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="7"/>
+      <c r="H58" s="13"/>
     </row>
     <row r="59" ht="16" customHeight="1" spans="1:8">
-      <c r="A59" s="22"/>
-      <c r="B59" s="22"/>
-      <c r="C59" s="22"/>
-      <c r="D59" s="22"/>
-      <c r="E59" s="22" t="s">
+      <c r="A59" s="12"/>
+      <c r="B59" s="12"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="F59" s="22"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="23"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="13"/>
     </row>
     <row r="60" ht="16" customHeight="1" spans="1:8">
-      <c r="A60" s="22"/>
-      <c r="B60" s="22" t="s">
+      <c r="A60" s="12"/>
+      <c r="B60" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="C60" s="22"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22" t="s">
+      <c r="C60" s="12"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="F60" s="22"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="23"/>
+      <c r="F60" s="12"/>
+      <c r="G60" s="7"/>
+      <c r="H60" s="13"/>
     </row>
     <row r="61" ht="16" customHeight="1" spans="1:8">
-      <c r="A61" s="22"/>
-      <c r="B61" s="22" t="s">
+      <c r="A61" s="12"/>
+      <c r="B61" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="C61" s="22"/>
-      <c r="D61" s="22"/>
-      <c r="E61" s="22" t="s">
+      <c r="C61" s="12"/>
+      <c r="D61" s="12"/>
+      <c r="E61" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="F61" s="22"/>
-      <c r="G61" s="19"/>
-      <c r="H61" s="23"/>
+      <c r="F61" s="12"/>
+      <c r="G61" s="7"/>
+      <c r="H61" s="13"/>
     </row>
     <row r="62" ht="16" customHeight="1" spans="1:8">
-      <c r="A62" s="22" t="s">
+      <c r="A62" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B62" s="22" t="s">
+      <c r="B62" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="C62" s="22"/>
-      <c r="D62" s="22"/>
-      <c r="E62" s="22" t="s">
+      <c r="C62" s="12"/>
+      <c r="D62" s="12"/>
+      <c r="E62" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="F62" s="22"/>
-      <c r="G62" s="19"/>
-      <c r="H62" s="23"/>
+      <c r="F62" s="12"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="13"/>
     </row>
     <row r="63" ht="16" customHeight="1" spans="1:8">
-      <c r="A63" s="22"/>
-      <c r="B63" s="22"/>
-      <c r="C63" s="22"/>
-      <c r="D63" s="22"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
-      <c r="G63" s="19"/>
-      <c r="H63" s="23"/>
+      <c r="A63" s="12"/>
+      <c r="B63" s="12"/>
+      <c r="C63" s="12"/>
+      <c r="D63" s="12"/>
+      <c r="E63" s="12"/>
+      <c r="F63" s="12"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="13"/>
     </row>
     <row r="64" ht="16" customHeight="1" spans="1:8">
-      <c r="A64" s="22"/>
-      <c r="B64" s="22"/>
-      <c r="C64" s="22"/>
-      <c r="D64" s="22"/>
-      <c r="E64" s="22" t="s">
+      <c r="A64" s="12"/>
+      <c r="B64" s="12"/>
+      <c r="C64" s="12"/>
+      <c r="D64" s="12"/>
+      <c r="E64" s="12" t="s">
         <v>204</v>
       </c>
-      <c r="F64" s="22"/>
-      <c r="G64" s="19"/>
-      <c r="H64" s="23"/>
+      <c r="F64" s="12"/>
+      <c r="G64" s="7"/>
+      <c r="H64" s="13"/>
     </row>
     <row r="65" ht="16" customHeight="1" spans="1:8">
-      <c r="A65" s="22"/>
-      <c r="B65" s="22"/>
-      <c r="C65" s="22"/>
-      <c r="D65" s="22" t="s">
+      <c r="A65" s="12"/>
+      <c r="B65" s="12"/>
+      <c r="C65" s="12"/>
+      <c r="D65" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="E65" s="22"/>
-      <c r="F65" s="22"/>
-      <c r="G65" s="19"/>
-      <c r="H65" s="23"/>
+      <c r="E65" s="12"/>
+      <c r="F65" s="12"/>
+      <c r="G65" s="7"/>
+      <c r="H65" s="13"/>
     </row>
     <row r="66" ht="16" customHeight="1" spans="1:8">
-      <c r="A66" s="22"/>
-      <c r="B66" s="22"/>
-      <c r="C66" s="22"/>
-      <c r="D66" s="22"/>
-      <c r="E66" s="22" t="s">
+      <c r="A66" s="12"/>
+      <c r="B66" s="12"/>
+      <c r="C66" s="12"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12" t="s">
         <v>206</v>
       </c>
-      <c r="F66" s="22"/>
-      <c r="G66" s="19"/>
-      <c r="H66" s="23"/>
+      <c r="F66" s="12"/>
+      <c r="G66" s="7"/>
+      <c r="H66" s="13"/>
     </row>
     <row r="67" ht="16" customHeight="1" spans="1:8">
-      <c r="A67" s="22" t="s">
+      <c r="A67" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B67" s="22" t="s">
+      <c r="B67" s="12" t="s">
         <v>207</v>
       </c>
-      <c r="C67" s="22"/>
-      <c r="D67" s="22"/>
-      <c r="E67" s="22" t="s">
+      <c r="C67" s="12"/>
+      <c r="D67" s="12"/>
+      <c r="E67" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="F67" s="22"/>
-      <c r="G67" s="19"/>
-      <c r="H67" s="23"/>
+      <c r="F67" s="12"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="13"/>
     </row>
     <row r="68" ht="16" customHeight="1" spans="1:8">
-      <c r="A68" s="22" t="s">
+      <c r="A68" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B68" s="22" t="s">
+      <c r="B68" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="C68" s="22"/>
-      <c r="D68" s="22"/>
-      <c r="E68" s="22" t="s">
+      <c r="C68" s="12"/>
+      <c r="D68" s="12"/>
+      <c r="E68" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="F68" s="22"/>
-      <c r="G68" s="19"/>
-      <c r="H68" s="23"/>
+      <c r="F68" s="12"/>
+      <c r="G68" s="7"/>
+      <c r="H68" s="13"/>
     </row>
     <row r="69" ht="16" customHeight="1" spans="1:8">
-      <c r="A69" s="22"/>
-      <c r="B69" s="22"/>
-      <c r="C69" s="22"/>
-      <c r="D69" s="22" t="s">
+      <c r="A69" s="12"/>
+      <c r="B69" s="12"/>
+      <c r="C69" s="12"/>
+      <c r="D69" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="E69" s="22"/>
-      <c r="F69" s="22"/>
-      <c r="G69" s="19"/>
-      <c r="H69" s="23"/>
+      <c r="E69" s="12"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="13"/>
     </row>
     <row r="70" ht="16" customHeight="1" spans="1:8">
-      <c r="A70" s="22"/>
-      <c r="B70" s="22"/>
-      <c r="C70" s="22"/>
-      <c r="D70" s="22"/>
-      <c r="E70" s="22" t="s">
+      <c r="A70" s="12"/>
+      <c r="B70" s="12"/>
+      <c r="C70" s="12"/>
+      <c r="D70" s="12"/>
+      <c r="E70" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="F70" s="22"/>
-      <c r="G70" s="19"/>
-      <c r="H70" s="23"/>
+      <c r="F70" s="12"/>
+      <c r="G70" s="7"/>
+      <c r="H70" s="13"/>
     </row>
     <row r="71" ht="16" customHeight="1" spans="1:8">
-      <c r="A71" s="22" t="s">
+      <c r="A71" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B71" s="22" t="s">
+      <c r="B71" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="C71" s="22"/>
-      <c r="D71" s="22"/>
-      <c r="E71" s="22" t="s">
+      <c r="C71" s="12"/>
+      <c r="D71" s="12"/>
+      <c r="E71" s="12" t="s">
         <v>214</v>
       </c>
-      <c r="F71" s="22" t="s">
+      <c r="F71" s="12" t="s">
         <v>215</v>
       </c>
-      <c r="G71" s="19"/>
-      <c r="H71" s="23"/>
+      <c r="G71" s="7"/>
+      <c r="H71" s="13"/>
     </row>
     <row r="72" ht="16" customHeight="1" spans="1:8">
-      <c r="A72" s="22"/>
-      <c r="B72" s="22"/>
-      <c r="C72" s="22"/>
-      <c r="D72" s="22"/>
-      <c r="E72" s="22" t="s">
+      <c r="A72" s="12"/>
+      <c r="B72" s="12"/>
+      <c r="C72" s="12"/>
+      <c r="D72" s="12"/>
+      <c r="E72" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="F72" s="22"/>
-      <c r="G72" s="19"/>
-      <c r="H72" s="23"/>
+      <c r="F72" s="12"/>
+      <c r="G72" s="7"/>
+      <c r="H72" s="13"/>
     </row>
     <row r="73" ht="16" customHeight="1" spans="1:8">
-      <c r="A73" s="22"/>
-      <c r="B73" s="22" t="s">
+      <c r="A73" s="12"/>
+      <c r="B73" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="C73" s="22"/>
-      <c r="D73" s="22"/>
-      <c r="E73" s="22" t="s">
+      <c r="C73" s="12"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="F73" s="22"/>
-      <c r="G73" s="19"/>
-      <c r="H73" s="23"/>
+      <c r="F73" s="12"/>
+      <c r="G73" s="7"/>
+      <c r="H73" s="13"/>
     </row>
     <row r="74" ht="16" customHeight="1" spans="1:8">
-      <c r="A74" s="22"/>
-      <c r="B74" s="22" t="s">
+      <c r="A74" s="12"/>
+      <c r="B74" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="C74" s="22"/>
-      <c r="D74" s="22"/>
-      <c r="E74" s="22" t="s">
+      <c r="C74" s="12"/>
+      <c r="D74" s="12"/>
+      <c r="E74" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="F74" s="22"/>
-      <c r="G74" s="19"/>
-      <c r="H74" s="23"/>
+      <c r="F74" s="12"/>
+      <c r="G74" s="7"/>
+      <c r="H74" s="13"/>
     </row>
     <row r="75" ht="16" customHeight="1" spans="1:8">
-      <c r="A75" s="22"/>
-      <c r="B75" s="22"/>
-      <c r="C75" s="22"/>
-      <c r="D75" s="22" t="s">
+      <c r="A75" s="12"/>
+      <c r="B75" s="12"/>
+      <c r="C75" s="12"/>
+      <c r="D75" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="E75" s="22"/>
-      <c r="F75" s="22"/>
-      <c r="G75" s="19"/>
-      <c r="H75" s="23"/>
+      <c r="E75" s="12"/>
+      <c r="F75" s="12"/>
+      <c r="G75" s="7"/>
+      <c r="H75" s="13"/>
     </row>
     <row r="76" spans="1:7">
-      <c r="A76" s="22"/>
-      <c r="B76" s="22"/>
-      <c r="C76" s="22"/>
-      <c r="D76" s="22"/>
-      <c r="E76" s="22" t="s">
+      <c r="A76" s="12"/>
+      <c r="B76" s="12"/>
+      <c r="C76" s="12"/>
+      <c r="D76" s="12"/>
+      <c r="E76" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="F76" s="22"/>
-      <c r="G76" s="24"/>
+      <c r="F76" s="12"/>
+      <c r="G76" s="14"/>
     </row>
     <row r="77" spans="1:7">
-      <c r="A77" s="22"/>
-      <c r="B77" s="22"/>
-      <c r="C77" s="22"/>
-      <c r="D77" s="22"/>
-      <c r="E77" s="22" t="s">
+      <c r="A77" s="12"/>
+      <c r="B77" s="12"/>
+      <c r="C77" s="12"/>
+      <c r="D77" s="12"/>
+      <c r="E77" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="F77" s="22"/>
-      <c r="G77" s="24"/>
+      <c r="F77" s="12"/>
+      <c r="G77" s="14"/>
     </row>
     <row r="78" spans="1:7">
-      <c r="A78" s="22"/>
-      <c r="B78" s="22"/>
-      <c r="C78" s="22" t="s">
+      <c r="A78" s="12"/>
+      <c r="B78" s="12"/>
+      <c r="C78" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="D78" s="22"/>
-      <c r="E78" s="22"/>
-      <c r="F78" s="22"/>
-      <c r="G78" s="24"/>
+      <c r="D78" s="12"/>
+      <c r="E78" s="12"/>
+      <c r="F78" s="12"/>
+      <c r="G78" s="14"/>
     </row>
     <row r="79" spans="1:6">
-      <c r="A79" s="22"/>
-      <c r="B79" s="22"/>
-      <c r="C79" s="22"/>
-      <c r="D79" s="22" t="s">
+      <c r="A79" s="12"/>
+      <c r="B79" s="12"/>
+      <c r="C79" s="12"/>
+      <c r="D79" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="E79" s="22"/>
-      <c r="F79" s="22"/>
+      <c r="E79" s="12"/>
+      <c r="F79" s="12"/>
     </row>
     <row r="80" spans="1:6">
-      <c r="A80" s="22"/>
-      <c r="B80" s="22"/>
-      <c r="C80" s="22"/>
-      <c r="D80" s="22"/>
-      <c r="E80" s="22" t="s">
+      <c r="A80" s="12"/>
+      <c r="B80" s="12"/>
+      <c r="C80" s="12"/>
+      <c r="D80" s="12"/>
+      <c r="E80" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="F80" s="22"/>
+      <c r="F80" s="12"/>
     </row>
     <row r="81" spans="1:6">
-      <c r="A81" s="22"/>
-      <c r="B81" s="22"/>
-      <c r="C81" s="22"/>
-      <c r="D81" s="22" t="s">
+      <c r="A81" s="12"/>
+      <c r="B81" s="12"/>
+      <c r="C81" s="12"/>
+      <c r="D81" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="E81" s="22"/>
-      <c r="F81" s="22"/>
+      <c r="E81" s="12"/>
+      <c r="F81" s="12"/>
     </row>
     <row r="82" spans="1:6">
-      <c r="A82" s="22"/>
-      <c r="B82" s="22"/>
-      <c r="C82" s="22"/>
-      <c r="D82" s="22"/>
-      <c r="E82" s="22" t="s">
+      <c r="A82" s="12"/>
+      <c r="B82" s="12"/>
+      <c r="C82" s="12"/>
+      <c r="D82" s="12"/>
+      <c r="E82" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="F82" s="22"/>
+      <c r="F82" s="12"/>
     </row>
     <row r="83" spans="1:6">
-      <c r="A83" s="22"/>
-      <c r="B83" s="22"/>
-      <c r="C83" s="22"/>
-      <c r="D83" s="22" t="s">
+      <c r="A83" s="12"/>
+      <c r="B83" s="12"/>
+      <c r="C83" s="12"/>
+      <c r="D83" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="E83" s="22"/>
-      <c r="F83" s="22"/>
+      <c r="E83" s="12"/>
+      <c r="F83" s="12"/>
     </row>
     <row r="84" spans="1:6">
-      <c r="A84" s="22"/>
-      <c r="B84" s="22"/>
-      <c r="C84" s="22"/>
-      <c r="D84" s="22"/>
-      <c r="E84" s="22" t="s">
+      <c r="A84" s="12"/>
+      <c r="B84" s="12"/>
+      <c r="C84" s="12"/>
+      <c r="D84" s="12"/>
+      <c r="E84" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="F84" s="22"/>
+      <c r="F84" s="12"/>
     </row>
     <row r="85" spans="1:6">
-      <c r="A85" s="22"/>
-      <c r="B85" s="22"/>
-      <c r="C85" s="22"/>
-      <c r="D85" s="22"/>
-      <c r="E85" s="22" t="s">
+      <c r="A85" s="12"/>
+      <c r="B85" s="12"/>
+      <c r="C85" s="12"/>
+      <c r="D85" s="12"/>
+      <c r="E85" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="F85" s="22"/>
+      <c r="F85" s="12"/>
     </row>
     <row r="86" spans="1:6">
-      <c r="A86" s="22"/>
-      <c r="B86" s="22"/>
-      <c r="C86" s="22" t="s">
+      <c r="A86" s="12"/>
+      <c r="B86" s="12"/>
+      <c r="C86" s="12" t="s">
         <v>232</v>
       </c>
-      <c r="D86" s="22"/>
-      <c r="E86" s="22"/>
-      <c r="F86" s="22"/>
+      <c r="D86" s="12"/>
+      <c r="E86" s="12"/>
+      <c r="F86" s="12"/>
     </row>
     <row r="87" spans="1:6">
-      <c r="A87" s="25"/>
-      <c r="B87" s="25"/>
-      <c r="C87" s="25"/>
-      <c r="D87" s="22" t="s">
+      <c r="A87" s="15"/>
+      <c r="B87" s="15"/>
+      <c r="C87" s="15"/>
+      <c r="D87" s="12" t="s">
         <v>233</v>
       </c>
-      <c r="E87" s="22"/>
-      <c r="F87" s="25"/>
+      <c r="E87" s="12"/>
+      <c r="F87" s="15"/>
     </row>
     <row r="88" spans="1:6">
-      <c r="A88" s="22"/>
-      <c r="B88" s="22"/>
-      <c r="C88" s="22"/>
-      <c r="D88" s="22" t="s">
+      <c r="A88" s="12"/>
+      <c r="B88" s="12"/>
+      <c r="C88" s="12"/>
+      <c r="D88" s="12" t="s">
         <v>234</v>
       </c>
-      <c r="E88" s="22"/>
-      <c r="F88" s="22"/>
+      <c r="E88" s="12"/>
+      <c r="F88" s="12"/>
     </row>
     <row r="89" spans="1:6">
-      <c r="A89" s="22"/>
-      <c r="B89" s="22"/>
-      <c r="C89" s="22"/>
-      <c r="D89" s="22" t="s">
+      <c r="A89" s="12"/>
+      <c r="B89" s="12"/>
+      <c r="C89" s="12"/>
+      <c r="D89" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="E89" s="22"/>
-      <c r="F89" s="22"/>
+      <c r="E89" s="12"/>
+      <c r="F89" s="12"/>
     </row>
     <row r="90" spans="1:6">
-      <c r="A90" s="22"/>
-      <c r="B90" s="22" t="s">
+      <c r="A90" s="12"/>
+      <c r="B90" s="12" t="s">
         <v>236</v>
       </c>
-      <c r="C90" s="22"/>
-      <c r="D90" s="22"/>
-      <c r="E90" s="22"/>
-      <c r="F90" s="22"/>
+      <c r="C90" s="12"/>
+      <c r="D90" s="12"/>
+      <c r="E90" s="12"/>
+      <c r="F90" s="12"/>
     </row>
     <row r="91" spans="1:6">
-      <c r="A91" s="22"/>
-      <c r="B91" s="22"/>
-      <c r="C91" s="22"/>
-      <c r="D91" s="22" t="s">
+      <c r="A91" s="12"/>
+      <c r="B91" s="12"/>
+      <c r="C91" s="12"/>
+      <c r="D91" s="12" t="s">
         <v>237</v>
       </c>
-      <c r="E91" s="22"/>
-      <c r="F91" s="22"/>
+      <c r="E91" s="12"/>
+      <c r="F91" s="12"/>
     </row>
     <row r="92" spans="1:6">
-      <c r="A92" s="22"/>
-      <c r="B92" s="22"/>
-      <c r="C92" s="22"/>
-      <c r="D92" s="22"/>
-      <c r="E92" s="22" t="s">
+      <c r="A92" s="12"/>
+      <c r="B92" s="12"/>
+      <c r="C92" s="12"/>
+      <c r="D92" s="12"/>
+      <c r="E92" s="12" t="s">
         <v>238</v>
       </c>
-      <c r="F92" s="22"/>
+      <c r="F92" s="12"/>
     </row>
     <row r="93" spans="1:6">
-      <c r="A93" s="22"/>
-      <c r="B93" s="22"/>
-      <c r="C93" s="22"/>
-      <c r="D93" s="22"/>
-      <c r="E93" s="22" t="s">
+      <c r="A93" s="12"/>
+      <c r="B93" s="12"/>
+      <c r="C93" s="12"/>
+      <c r="D93" s="12"/>
+      <c r="E93" s="12" t="s">
         <v>239</v>
       </c>
-      <c r="F93" s="22"/>
+      <c r="F93" s="12"/>
     </row>
     <row r="94" spans="1:6">
-      <c r="A94" s="22"/>
-      <c r="B94" s="22"/>
-      <c r="C94" s="22"/>
-      <c r="D94" s="22" t="s">
+      <c r="A94" s="12"/>
+      <c r="B94" s="12"/>
+      <c r="C94" s="12"/>
+      <c r="D94" s="12" t="s">
         <v>240</v>
       </c>
-      <c r="E94" s="22"/>
-      <c r="F94" s="22"/>
+      <c r="E94" s="12"/>
+      <c r="F94" s="12"/>
     </row>
     <row r="95" spans="1:6">
-      <c r="A95" s="22"/>
-      <c r="B95" s="22"/>
-      <c r="C95" s="22"/>
-      <c r="D95" s="22" t="s">
+      <c r="A95" s="12"/>
+      <c r="B95" s="12"/>
+      <c r="C95" s="12"/>
+      <c r="D95" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="E95" s="22"/>
-      <c r="F95" s="22"/>
+      <c r="E95" s="12"/>
+      <c r="F95" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4324,157 +3841,157 @@
   <dimension ref="A1:H99"/>
   <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="13" customHeight="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="24.9153846153846" style="13" customWidth="1"/>
-    <col min="2" max="2" width="19.8307692307692" style="13" customWidth="1"/>
-    <col min="3" max="3" width="2.66923076923077" style="13" customWidth="1"/>
-    <col min="4" max="4" width="3.83076923076923" style="13" customWidth="1"/>
-    <col min="5" max="5" width="14.4153846153846" style="13" customWidth="1"/>
-    <col min="6" max="6" width="12.1692307692308" style="13" customWidth="1"/>
-    <col min="7" max="8" width="4.5" style="13" customWidth="1"/>
-    <col min="9" max="16384" width="8.66923076923077" style="13"/>
+    <col min="1" max="1" width="24.9153846153846" style="4" customWidth="1"/>
+    <col min="2" max="2" width="19.8307692307692" style="4" customWidth="1"/>
+    <col min="3" max="3" width="2.66923076923077" style="4" customWidth="1"/>
+    <col min="4" max="4" width="3.83076923076923" style="4" customWidth="1"/>
+    <col min="5" max="5" width="14.4153846153846" style="4" customWidth="1"/>
+    <col min="6" max="6" width="12.1692307692308" style="4" customWidth="1"/>
+    <col min="7" max="8" width="4.5" style="4" customWidth="1"/>
+    <col min="9" max="16384" width="8.66923076923077" style="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="14" customHeight="1" spans="2:2">
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="4" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:8">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" customHeight="1" spans="2:7">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="G3" s="17"/>
+      <c r="G3" s="5"/>
     </row>
     <row r="4" customHeight="1" spans="3:7">
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="G4" s="17"/>
+      <c r="G4" s="5"/>
     </row>
     <row r="5" customHeight="1" spans="3:7">
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="G5" s="17"/>
+      <c r="G5" s="5"/>
     </row>
     <row r="6" customHeight="1" spans="3:7">
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="G6" s="17"/>
+      <c r="G6" s="5"/>
     </row>
     <row r="7" customHeight="1" spans="2:3">
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="7" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="8" customHeight="1" spans="2:3">
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="7" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="9" customHeight="1" spans="2:3">
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="7" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="10" customHeight="1" spans="3:3">
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="7" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="11" customHeight="1" spans="3:3">
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="7" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="12" customHeight="1" spans="1:3">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="7" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="13" customHeight="1" spans="2:3">
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="7" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="14" customHeight="1" spans="3:3">
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="7" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="15" customHeight="1" spans="3:3">
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="7" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="5:5">
-      <c r="E17" s="17"/>
+      <c r="E17" s="5"/>
     </row>
     <row r="19" customHeight="1" spans="2:3">
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="4" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="21" customHeight="1" spans="1:3">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="4" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="22" customHeight="1" spans="4:4">
-      <c r="D22" s="20" t="s">
+      <c r="D22" s="8" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="26" customHeight="1" spans="2:2">
-      <c r="B26" s="21"/>
+      <c r="B26" s="9"/>
     </row>
     <row r="47" customHeight="1" spans="4:4">
       <c r="D47" s="10"/>
@@ -4552,7 +4069,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="7:7">
-      <c r="G1" s="11"/>
+      <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
@@ -4567,7 +4084,7 @@
       <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -4582,308 +4099,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:I34"/>
-  <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="14"/>
-  <cols>
-    <col min="1" max="1" width="25.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.8307692307692" style="1" customWidth="1"/>
-    <col min="3" max="3" width="2.41538461538462" style="1" customWidth="1"/>
-    <col min="4" max="4" width="3.33076923076923" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6692307692308" style="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1692307692308" style="1" customWidth="1"/>
-    <col min="7" max="7" width="4.5" style="16" customWidth="1"/>
-    <col min="8" max="8" width="4.5" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.66923076923077" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:2">
-      <c r="B1" s="1" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="9"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-    </row>
-    <row r="29" ht="15.5" spans="1:5">
-      <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29"/>
-    </row>
-    <row r="30" ht="15.5" spans="1:9">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30"/>
-      <c r="I30" s="10"/>
-    </row>
-    <row r="31" ht="15.5" spans="1:9">
-      <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10"/>
-    </row>
-    <row r="32" ht="15.5" spans="1:9">
-      <c r="A32"/>
-      <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="H32" s="10"/>
-      <c r="I32" s="10"/>
-    </row>
-    <row r="33" ht="15.5" spans="1:9">
-      <c r="A33"/>
-      <c r="B33"/>
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="10"/>
-    </row>
-    <row r="34" spans="8:9">
-      <c r="H34" s="10"/>
-      <c r="I34" s="10"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="B1:H41"/>
-  <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="14" outlineLevelCol="7"/>
-  <cols>
-    <col min="1" max="1" width="25.4153846153846" style="13" customWidth="1"/>
-    <col min="2" max="2" width="19.8307692307692" style="13" customWidth="1"/>
-    <col min="3" max="3" width="5.66923076923077" style="13" customWidth="1"/>
-    <col min="4" max="4" width="7.08461538461538" style="13" customWidth="1"/>
-    <col min="5" max="5" width="7.75384615384615" style="13" customWidth="1"/>
-    <col min="6" max="6" width="12.1692307692308" style="13" customWidth="1"/>
-    <col min="7" max="7" width="4.5" style="14" customWidth="1"/>
-    <col min="8" max="8" width="4.5" style="13" customWidth="1"/>
-    <col min="9" max="16384" width="8.66923076923077" style="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:2">
-      <c r="B1" s="13" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="2" spans="2:8">
-      <c r="B2" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="3:5">
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-    </row>
-    <row r="4" spans="3:5">
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-    </row>
-    <row r="5" spans="3:5">
-      <c r="C5" s="10"/>
-      <c r="E5" s="10"/>
-    </row>
-    <row r="6" spans="3:5">
-      <c r="C6" s="10"/>
-      <c r="E6" s="10"/>
-    </row>
-    <row r="7" spans="3:5">
-      <c r="C7" s="10"/>
-      <c r="E7" s="10"/>
-    </row>
-    <row r="8" spans="3:5">
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-    </row>
-    <row r="10" spans="4:4">
-      <c r="D10" s="10"/>
-    </row>
-    <row r="11" spans="4:4">
-      <c r="D11" s="10"/>
-    </row>
-    <row r="12" spans="4:4">
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="4:4">
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="4:4">
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="4:4">
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="4:4">
-      <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="4:4">
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="4:4">
-      <c r="D18" s="1"/>
-    </row>
-    <row r="35" spans="3:4">
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-    </row>
-    <row r="36" spans="3:4">
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-    </row>
-    <row r="37" spans="3:4">
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-    </row>
-    <row r="38" spans="3:4">
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-    </row>
-    <row r="39" spans="3:4">
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-    </row>
-    <row r="40" spans="3:4">
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-    </row>
-    <row r="41" spans="3:4">
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="142" orientation="portrait"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A2:H5"/>
@@ -4912,7 +4127,7 @@
       <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -4921,17 +4136,17 @@
     </row>
     <row r="3" ht="14.75" spans="3:3">
       <c r="C3" s="1" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="4" ht="14.75" spans="4:4">
+      <c r="D4" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="5" ht="14.75" spans="4:4">
+      <c r="D5" s="3" t="s">
         <v>270</v>
-      </c>
-    </row>
-    <row r="4" ht="14.75" spans="4:4">
-      <c r="D4" s="12" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="5" ht="14.75" spans="4:4">
-      <c r="D5" s="12" t="s">
-        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -4939,18 +4154,4 @@
   <pageSetup paperSize="142" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5"/>
-  <cols>
-    <col min="1" max="16384" width="8.66923076923077" style="8"/>
-  </cols>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
py + ploty iint
</commit_message>
<xml_diff>
--- a/p/py-25/py-libs/pandas/topic-list_pandas.xlsx
+++ b/p/py-25/py-libs/pandas/topic-list_pandas.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="381">
   <si>
     <t>Dataframe: Two dimensional Data Structure, like table</t>
   </si>
@@ -88,15 +88,6 @@
     <t>topic</t>
   </si>
   <si>
-    <t>sub-topic</t>
-  </si>
-  <si>
-    <t>priority</t>
-  </si>
-  <si>
-    <t>flag</t>
-  </si>
-  <si>
     <t>basic data monitoring</t>
   </si>
   <si>
@@ -295,10 +286,7 @@
     <t>apply(float)</t>
   </si>
   <si>
-    <t>row wise</t>
-  </si>
-  <si>
-    <t>applymap works element wise on df</t>
+    <t>row wise, applymap works element wise on df</t>
   </si>
   <si>
     <t>stackoverflow.com/questions/19798153/difference-between-map-applymap-and-apply-methods-in-pandas</t>
@@ -663,10 +651,7 @@
     <t>left, right, outer, inner, cross</t>
   </si>
   <si>
-    <t>how</t>
-  </si>
-  <si>
-    <t>pd.merge(data1, data2, on='subject_id', how='outer')</t>
+    <t>how,  pd.merge(data1, data2, on='subject_id', how='outer')</t>
   </si>
   <si>
     <t>merge(left_d, right_d, on="col1")</t>
@@ -758,13 +743,11 @@
     <t>.groupBy('colName')</t>
   </si>
   <si>
-    <t>// not similar to sql</t>
-  </si>
-  <si>
     <t>Data-Analysis-with-Pandas-and-Python-master\GroupBy.ipynb</t>
   </si>
   <si>
-    <t>.groupBy is very agile method, described in detail here</t>
+    <t>// not similar to sql
+.groupBy is very agile method, described in detail here</t>
   </si>
   <si>
     <t>pandas_exercises-master\01_Getting_&amp;_Knowing_Your_Data\Chipotle\Exercise_with_Solutions.ipynb</t>
@@ -859,6 +842,15 @@
   </si>
   <si>
     <t>Most basic and few extra things in py</t>
+  </si>
+  <si>
+    <t>sub-topic</t>
+  </si>
+  <si>
+    <t>priority</t>
+  </si>
+  <si>
+    <t>flag</t>
   </si>
   <si>
     <t>Basic operations</t>
@@ -2216,7 +2208,9 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -2659,16 +2653,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H171"/>
+  <dimension ref="A1:H168"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="27.3307692307692" style="25" customWidth="1"/>
     <col min="2" max="2" width="19.8307692307692" style="25" customWidth="1"/>
-    <col min="3" max="3" width="2.41538461538462" style="26" customWidth="1"/>
-    <col min="4" max="4" width="3.33076923076923" style="26" customWidth="1"/>
-    <col min="5" max="5" width="8.89230769230769" style="25" customWidth="1"/>
-    <col min="6" max="6" width="12.1692307692308" style="25" customWidth="1"/>
-    <col min="7" max="8" width="4.5" style="25" customWidth="1"/>
+    <col min="3" max="4" width="2.53846153846154" style="26" customWidth="1"/>
+    <col min="5" max="7" width="2.53846153846154" style="25" customWidth="1"/>
+    <col min="8" max="8" width="48.4230769230769" style="25" customWidth="1"/>
     <col min="9" max="16384" width="11" style="25"/>
   </cols>
   <sheetData>
@@ -2677,7 +2669,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:7">
       <c r="A2" s="25" t="s">
         <v>15</v>
       </c>
@@ -2687,398 +2679,396 @@
       <c r="C2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" s="25" t="s">
-        <v>20</v>
-      </c>
+      <c r="G2" s="27"/>
     </row>
     <row r="3" spans="3:7">
       <c r="C3" s="26" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G3" s="27"/>
     </row>
     <row r="4" ht="12" customHeight="1" spans="2:7">
       <c r="B4" s="25" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G4" s="27"/>
     </row>
     <row r="5" spans="7:7">
       <c r="G5" s="27"/>
     </row>
-    <row r="6" spans="7:7">
+    <row r="6" spans="3:7">
+      <c r="C6" s="26" t="s">
+        <v>21</v>
+      </c>
       <c r="G6" s="27"/>
     </row>
-    <row r="7" spans="7:7">
+    <row r="7" spans="4:7">
+      <c r="D7" s="26" t="s">
+        <v>22</v>
+      </c>
       <c r="G7" s="27"/>
     </row>
-    <row r="8" spans="7:7">
+    <row r="8" spans="2:7">
+      <c r="B8" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>24</v>
+      </c>
       <c r="G8" s="27"/>
     </row>
-    <row r="9" spans="3:7">
-      <c r="C9" s="26" t="s">
-        <v>24</v>
+    <row r="9" spans="5:7">
+      <c r="E9" s="25" t="s">
+        <v>25</v>
       </c>
       <c r="G9" s="27"/>
     </row>
-    <row r="10" spans="4:7">
-      <c r="D10" s="26" t="s">
-        <v>25</v>
+    <row r="10" spans="5:7">
+      <c r="E10" s="25" t="s">
+        <v>26</v>
       </c>
       <c r="G10" s="27"/>
     </row>
     <row r="11" spans="2:7">
       <c r="B11" s="25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G11" s="27"/>
     </row>
-    <row r="12" spans="5:7">
+    <row r="12" spans="2:7">
+      <c r="B12" s="25" t="s">
+        <v>29</v>
+      </c>
       <c r="E12" s="25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G12" s="27"/>
     </row>
-    <row r="13" spans="5:7">
+    <row r="13" spans="1:7">
+      <c r="A13" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>32</v>
+      </c>
       <c r="E13" s="25" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="G13" s="27"/>
     </row>
-    <row r="14" spans="2:7">
-      <c r="B14" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="E14" s="25" t="s">
-        <v>31</v>
+    <row r="14" spans="6:7">
+      <c r="F14" s="25" t="s">
+        <v>34</v>
       </c>
       <c r="G14" s="27"/>
     </row>
-    <row r="15" spans="2:7">
-      <c r="B15" s="25" t="s">
-        <v>32</v>
-      </c>
+    <row r="15" spans="5:7">
       <c r="E15" s="25" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G15" s="27"/>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="25" t="s">
+    <row r="16" spans="4:7">
+      <c r="D16" s="26" t="s">
         <v>36</v>
       </c>
       <c r="G16" s="27"/>
     </row>
-    <row r="17" spans="6:7">
-      <c r="F17" s="25" t="s">
+    <row r="17" spans="5:7">
+      <c r="E17" s="25" t="s">
         <v>37</v>
       </c>
       <c r="G17" s="27"/>
     </row>
-    <row r="18" spans="5:7">
+    <row r="18" spans="1:7">
+      <c r="A18" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>39</v>
+      </c>
       <c r="E18" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" s="27"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="G18" s="27"/>
-    </row>
-    <row r="19" spans="4:7">
-      <c r="D19" s="26" t="s">
-        <v>39</v>
+      <c r="B19" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="25" t="s">
+        <v>42</v>
       </c>
       <c r="G19" s="27"/>
     </row>
-    <row r="20" spans="5:7">
-      <c r="E20" s="25" t="s">
-        <v>40</v>
+    <row r="20" spans="4:7">
+      <c r="D20" s="26" t="s">
+        <v>43</v>
       </c>
       <c r="G20" s="27"/>
     </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" s="25" t="s">
-        <v>42</v>
-      </c>
+    <row r="21" spans="5:7">
       <c r="E21" s="25" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G21" s="27"/>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="25" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="F22" s="25" t="s">
+        <v>47</v>
       </c>
       <c r="G22" s="27"/>
     </row>
-    <row r="23" spans="4:7">
-      <c r="D23" s="26" t="s">
-        <v>46</v>
+    <row r="23" spans="1:7">
+      <c r="A23" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="E23" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="F23" s="25" t="s">
+        <v>50</v>
       </c>
       <c r="G23" s="27"/>
     </row>
-    <row r="24" spans="5:7">
+    <row r="24" spans="2:7">
+      <c r="B24" s="25" t="s">
+        <v>51</v>
+      </c>
       <c r="E24" s="25" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G24" s="27"/>
     </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="25" t="s">
-        <v>41</v>
-      </c>
+    <row r="25" spans="2:7">
       <c r="B25" s="25" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="F25" s="25" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G25" s="27"/>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="25" t="s">
-        <v>51</v>
+        <v>55</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>56</v>
       </c>
       <c r="E26" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="F26" s="25" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G26" s="27"/>
     </row>
-    <row r="27" spans="2:7">
-      <c r="B27" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="E27" s="25" t="s">
-        <v>55</v>
+    <row r="27" spans="6:7">
+      <c r="F27" s="25" t="s">
+        <v>58</v>
       </c>
       <c r="G27" s="27"/>
     </row>
-    <row r="28" spans="2:7">
-      <c r="B28" s="25" t="s">
-        <v>56</v>
-      </c>
+    <row r="28" spans="5:7">
       <c r="E28" s="25" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G28" s="27"/>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="B29" s="25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E29" s="25" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G29" s="27"/>
     </row>
-    <row r="30" spans="6:7">
-      <c r="F30" s="25" t="s">
-        <v>61</v>
+    <row r="30" spans="1:7">
+      <c r="A30" s="25" t="s">
+        <v>62</v>
       </c>
       <c r="G30" s="27"/>
     </row>
-    <row r="31" spans="5:7">
-      <c r="E31" s="25" t="s">
-        <v>62</v>
-      </c>
+    <row r="31" spans="7:7">
       <c r="G31" s="27"/>
     </row>
-    <row r="32" spans="1:7">
-      <c r="A32" s="25" t="s">
+    <row r="32" spans="4:7">
+      <c r="D32" s="26" t="s">
         <v>63</v>
-      </c>
-      <c r="E32" s="25" t="s">
-        <v>64</v>
       </c>
       <c r="G32" s="27"/>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="F33" s="25" t="s">
         <v>65</v>
       </c>
       <c r="G33" s="27"/>
     </row>
-    <row r="34" spans="7:7">
+    <row r="34" spans="7:8">
       <c r="G34" s="27"/>
-    </row>
-    <row r="35" spans="4:7">
-      <c r="D35" s="26" t="s">
+      <c r="H34" s="25" t="s">
         <v>66</v>
       </c>
+    </row>
+    <row r="35" spans="7:8">
       <c r="G35" s="27"/>
-    </row>
-    <row r="36" spans="1:7">
+      <c r="H35" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E36" s="25" t="s">
         <v>68</v>
       </c>
       <c r="G36" s="27"/>
-    </row>
-    <row r="37" spans="5:7">
-      <c r="E37" s="25" t="s">
+      <c r="H36" s="25" t="s">
         <v>69</v>
       </c>
+    </row>
+    <row r="37" spans="4:7">
+      <c r="D37" s="26" t="s">
+        <v>70</v>
+      </c>
       <c r="G37" s="27"/>
     </row>
-    <row r="38" spans="5:7">
-      <c r="E38" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="G38" s="27"/>
-    </row>
-    <row r="39" spans="1:7">
-      <c r="A39" s="25" t="s">
+    <row r="38" spans="3:3">
+      <c r="C38" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="E39" s="25" t="s">
+    </row>
+    <row r="39" spans="4:4">
+      <c r="D39" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="G39" s="27"/>
-    </row>
-    <row r="40" spans="4:7">
-      <c r="D40" s="26" t="s">
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="E40" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="G40" s="27"/>
-    </row>
-    <row r="41" spans="3:3">
-      <c r="C41" s="26" t="s">
+    </row>
+    <row r="41" spans="5:5">
+      <c r="E41" s="25" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="4:4">
-      <c r="D42" s="26" t="s">
+    <row r="42" spans="5:5">
+      <c r="E42" s="25" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="25" t="s">
-        <v>41</v>
+        <v>76</v>
       </c>
       <c r="E43" s="25" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="5:5">
       <c r="E44" s="25" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="45" spans="5:5">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="25" t="s">
+        <v>79</v>
+      </c>
       <c r="E45" s="25" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5">
-      <c r="A46" s="25" t="s">
-        <v>79</v>
-      </c>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="46" spans="5:5">
       <c r="E46" s="25" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="47" spans="5:5">
-      <c r="E47" s="25" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
-      <c r="A48" s="25" t="s">
+    <row r="48" spans="2:6">
+      <c r="B48" s="28" t="s">
         <v>82</v>
       </c>
       <c r="E48" s="25" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="49" spans="5:5">
-      <c r="E49" s="25" t="s">
+      <c r="F48" s="25" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="51" spans="2:7">
-      <c r="B51" s="28" t="s">
+    <row r="49" spans="1:1">
+      <c r="A49" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="E51" s="25" t="s">
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="E50" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="F51" s="25" t="s">
+    </row>
+    <row r="51" spans="5:5">
+      <c r="E51" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="G51" s="25" t="s">
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" s="25" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="52" spans="1:1">
-      <c r="A52" s="29" t="s">
+      <c r="C53" s="26" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
-      <c r="A53" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="E53" s="25" t="s">
+    <row r="54" spans="4:4">
+      <c r="D54" s="26" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="54" spans="5:5">
-      <c r="E54" s="30" t="s">
+    <row r="55" spans="1:5">
+      <c r="A55" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B55" s="25" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="A56" s="25" t="s">
+      <c r="E55" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="C56" s="26" t="s">
+    </row>
+    <row r="56" spans="4:4">
+      <c r="D56" s="26" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="57" spans="4:4">
-      <c r="D57" s="26" t="s">
+    <row r="57" spans="5:5">
+      <c r="E57" s="25" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
-      <c r="A58" s="25" t="s">
-        <v>41</v>
-      </c>
+    <row r="58" spans="2:5">
       <c r="B58" s="25" t="s">
         <v>95</v>
       </c>
@@ -3086,69 +3076,72 @@
         <v>96</v>
       </c>
     </row>
-    <row r="59" spans="4:4">
-      <c r="D59" s="26" t="s">
+    <row r="59" spans="5:5">
+      <c r="E59" s="25" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="60" spans="5:5">
-      <c r="E60" s="25" t="s">
+    <row r="60" spans="4:4">
+      <c r="D60" s="26" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="61" spans="2:5">
-      <c r="B61" s="25" t="s">
+    <row r="61" spans="4:4">
+      <c r="D61" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="E61" s="25" t="s">
+    </row>
+    <row r="62" spans="4:4">
+      <c r="D62" s="26" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="62" spans="5:5">
-      <c r="E62" s="25" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="63" spans="4:4">
       <c r="D63" s="26" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" s="25" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="64" spans="4:4">
-      <c r="D64" s="26" t="s">
+      <c r="E64" s="25" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="65" spans="4:4">
-      <c r="D65" s="26" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="66" spans="4:4">
       <c r="D66" s="26" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="67" spans="4:4">
+      <c r="D67" s="26" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
-      <c r="A67" s="25" t="s">
+    <row r="68" spans="5:5">
+      <c r="E68" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="E67" s="25" t="s">
+    </row>
+    <row r="69" spans="5:5">
+      <c r="E69" s="25" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="69" spans="4:4">
-      <c r="D69" s="26" t="s">
+    <row r="70" spans="1:5">
+      <c r="A70" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B70" s="25" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="70" spans="4:4">
-      <c r="D70" s="26" t="s">
+      <c r="E70" s="25" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="71" spans="5:5">
-      <c r="E71" s="25" t="s">
+    <row r="71" spans="4:4">
+      <c r="D71" s="26" t="s">
         <v>110</v>
       </c>
     </row>
@@ -3157,35 +3150,37 @@
         <v>111</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
-      <c r="A73" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B73" s="25" t="s">
+    <row r="73" spans="5:5">
+      <c r="E73" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="E73" s="25" t="s">
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="30"/>
+      <c r="B75" s="30"/>
+      <c r="E75" s="25" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="74" spans="4:4">
-      <c r="D74" s="26" t="s">
+    <row r="76" spans="1:5">
+      <c r="A76" s="30"/>
+      <c r="B76" s="30"/>
+      <c r="E76" s="25" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="75" spans="5:5">
-      <c r="E75" s="25" t="s">
+    <row r="77" spans="1:5">
+      <c r="A77" s="30"/>
+      <c r="B77" s="30"/>
+      <c r="E77" s="25" t="s">
         <v>115</v>
-      </c>
-    </row>
-    <row r="76" spans="5:5">
-      <c r="E76" s="25" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" s="30"/>
-      <c r="B78" s="30"/>
+      <c r="B78" s="25" t="s">
+        <v>116</v>
+      </c>
       <c r="E78" s="25" t="s">
         <v>117</v>
       </c>
@@ -3197,15 +3192,19 @@
         <v>118</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
-      <c r="A80" s="30"/>
+    <row r="80" spans="1:6">
+      <c r="A80" s="25" t="s">
+        <v>102</v>
+      </c>
       <c r="B80" s="30"/>
-      <c r="E80" s="25" t="s">
+      <c r="F80" s="25" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="81" spans="1:5">
-      <c r="A81" s="30"/>
+      <c r="A81" s="25" t="s">
+        <v>38</v>
+      </c>
       <c r="B81" s="25" t="s">
         <v>120</v>
       </c>
@@ -3213,651 +3212,618 @@
         <v>121</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
-      <c r="A82" s="30"/>
-      <c r="B82" s="30"/>
+    <row r="82" spans="2:5">
+      <c r="B82" s="25" t="s">
+        <v>122</v>
+      </c>
       <c r="E82" s="25" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6">
-      <c r="A83" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="B83" s="30"/>
-      <c r="F83" s="25" t="s">
         <v>123</v>
+      </c>
+    </row>
+    <row r="83" spans="5:5">
+      <c r="E83" s="25" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" s="25" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B84" s="25" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E84" s="25" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="85" spans="2:5">
-      <c r="B85" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="E85" s="25" t="s">
+    </row>
+    <row r="85" spans="1:4">
+      <c r="A85" s="30"/>
+      <c r="D85" s="26" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="86" spans="5:5">
+    <row r="86" spans="1:5">
+      <c r="A86" s="30"/>
+      <c r="B86" s="25" t="s">
+        <v>128</v>
+      </c>
       <c r="E86" s="25" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="87" spans="1:5">
-      <c r="A87" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B87" s="25" t="s">
-        <v>129</v>
+      <c r="A87" s="30" t="s">
+        <v>130</v>
       </c>
       <c r="E87" s="25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="30"/>
       <c r="D88" s="26" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5">
-      <c r="A89" s="30"/>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="89" spans="2:5">
       <c r="B89" s="25" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E89" s="25" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="90" spans="1:5">
-      <c r="A90" s="30" t="s">
+      <c r="A90" s="25" t="s">
         <v>134</v>
       </c>
       <c r="E90" s="25" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="91" spans="1:4">
-      <c r="A91" s="30"/>
-      <c r="D91" s="26" t="s">
+    <row r="91" spans="6:6">
+      <c r="F91" s="25" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="92" spans="2:5">
-      <c r="B92" s="25" t="s">
-        <v>132</v>
-      </c>
+    <row r="92" spans="5:5">
       <c r="E92" s="25" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
-      <c r="A93" s="25" t="s">
+    <row r="94" spans="1:4">
+      <c r="A94" s="30"/>
+      <c r="D94" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="E93" s="25" t="s">
+    </row>
+    <row r="95" spans="2:5">
+      <c r="B95" s="25" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="94" spans="6:6">
-      <c r="F94" s="25" t="s">
+      <c r="E95" s="25" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="95" spans="5:5">
-      <c r="E95" s="25" t="s">
+    <row r="96" spans="2:2">
+      <c r="B96" s="25" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="97" spans="1:4">
-      <c r="A97" s="30"/>
-      <c r="D97" s="26" t="s">
+    <row r="97" spans="5:5">
+      <c r="E97" s="25" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="98" spans="2:5">
-      <c r="B98" s="25" t="s">
+    <row r="98" spans="6:6">
+      <c r="F98" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="E98" s="25" t="s">
+    </row>
+    <row r="99" spans="6:6">
+      <c r="F99" s="25" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="99" spans="2:2">
-      <c r="B99" s="25" t="s">
+    <row r="100" spans="6:6">
+      <c r="F100" s="25" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="100" spans="5:5">
-      <c r="E100" s="25" t="s">
+    <row r="101" spans="4:4">
+      <c r="D101" s="26" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="101" spans="6:6">
-      <c r="F101" s="25" t="s">
+    <row r="102" spans="1:5">
+      <c r="A102" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B102" s="25" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="102" spans="6:6">
-      <c r="F102" s="25" t="s">
+      <c r="E102" s="25" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="103" spans="6:6">
-      <c r="F103" s="25" t="s">
+    <row r="103" spans="1:2">
+      <c r="A103" s="25" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="104" spans="4:4">
-      <c r="D104" s="26" t="s">
+      <c r="B103" s="25" t="s">
         <v>150</v>
+      </c>
+    </row>
+    <row r="104" spans="2:2">
+      <c r="B104" s="25" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="105" spans="1:5">
       <c r="A105" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B105" s="25" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E105" s="25" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="106" spans="1:2">
-      <c r="A106" s="25" t="s">
+    <row r="106" spans="2:6">
+      <c r="B106" s="25" t="s">
         <v>153</v>
       </c>
-      <c r="B106" s="25" t="s">
+      <c r="F106" s="25" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="2:4">
       <c r="B107" s="25" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="108" spans="1:5">
-      <c r="A108" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="E108" s="25" t="s">
+      <c r="D107" s="26" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="109" spans="2:6">
-      <c r="B109" s="25" t="s">
+    <row r="108" spans="2:2">
+      <c r="B108" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="F109" s="25" t="s">
+    </row>
+    <row r="109" spans="5:5">
+      <c r="E109" s="25" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="110" spans="2:4">
+    <row r="110" spans="1:5">
+      <c r="A110" s="25" t="s">
+        <v>159</v>
+      </c>
       <c r="B110" s="25" t="s">
+        <v>160</v>
+      </c>
+      <c r="E110" s="31" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5">
+      <c r="A111" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="D110" s="26" t="s">
+      <c r="B111" s="25" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="111" spans="2:2">
-      <c r="B111" s="25" t="s">
-        <v>161</v>
+      <c r="E111" s="31" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="112" spans="5:5">
-      <c r="E112" s="25" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5">
-      <c r="A113" s="25" t="s">
+      <c r="E112" s="32" t="s">
         <v>163</v>
       </c>
-      <c r="B113" s="25" t="s">
+    </row>
+    <row r="114" spans="4:4">
+      <c r="D114" s="26" t="s">
         <v>164</v>
       </c>
-      <c r="E113" s="31" t="s">
+    </row>
+    <row r="115" spans="1:6">
+      <c r="A115" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B115" s="25" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="114" spans="1:5">
-      <c r="A114" s="25" t="s">
-        <v>163</v>
-      </c>
-      <c r="B114" s="25" t="s">
-        <v>164</v>
-      </c>
-      <c r="E114" s="31" t="s">
+      <c r="C115" s="28"/>
+      <c r="D115" s="28"/>
+      <c r="E115" s="30"/>
+      <c r="F115" s="30" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="115" spans="5:5">
-      <c r="E115" s="32" t="s">
+    <row r="116" spans="2:6">
+      <c r="B116" s="25" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="117" spans="4:4">
-      <c r="D117" s="26" t="s">
+      <c r="C116" s="28"/>
+      <c r="D116" s="28"/>
+      <c r="E116" s="30"/>
+      <c r="F116" s="30"/>
+    </row>
+    <row r="117" spans="3:6">
+      <c r="C117" s="28"/>
+      <c r="D117" s="28"/>
+      <c r="E117" s="30"/>
+      <c r="F117" s="30"/>
+    </row>
+    <row r="118" spans="2:6">
+      <c r="B118" s="25" t="s">
         <v>168</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6">
-      <c r="A118" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B118" s="25" t="s">
-        <v>169</v>
       </c>
       <c r="C118" s="28"/>
       <c r="D118" s="28"/>
-      <c r="E118" s="30"/>
-      <c r="F118" s="30" t="s">
-        <v>170</v>
-      </c>
+      <c r="E118" s="25" t="s">
+        <v>169</v>
+      </c>
+      <c r="F118" s="30"/>
     </row>
     <row r="119" spans="2:6">
       <c r="B119" s="25" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C119" s="28"/>
       <c r="D119" s="28"/>
       <c r="E119" s="30"/>
       <c r="F119" s="30"/>
     </row>
-    <row r="120" spans="3:6">
-      <c r="C120" s="28"/>
-      <c r="D120" s="28"/>
-      <c r="E120" s="30"/>
-      <c r="F120" s="30"/>
-    </row>
-    <row r="121" spans="2:6">
+    <row r="120" spans="4:5">
+      <c r="D120" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="E120" s="26"/>
+    </row>
+    <row r="121" spans="1:5">
+      <c r="A121" s="25" t="s">
+        <v>172</v>
+      </c>
       <c r="B121" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="C121" s="28"/>
-      <c r="D121" s="28"/>
-      <c r="E121" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="F121" s="30"/>
+      <c r="E121" s="26" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="122" spans="2:6">
       <c r="B122" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="C122" s="28"/>
-      <c r="D122" s="28"/>
-      <c r="E122" s="30"/>
-      <c r="F122" s="30"/>
-    </row>
-    <row r="123" spans="4:5">
-      <c r="D123" s="26" t="s">
         <v>175</v>
       </c>
-      <c r="E123" s="26"/>
+      <c r="E122" s="26"/>
+      <c r="F122" s="25" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="123" spans="5:5">
+      <c r="E123" s="33" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="124" spans="1:5">
-      <c r="A124" s="25" t="s">
-        <v>176</v>
-      </c>
-      <c r="B124" s="25" t="s">
-        <v>177</v>
-      </c>
-      <c r="E124" s="26" t="s">
+      <c r="A124" s="29" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="125" spans="2:7">
-      <c r="B125" s="25" t="s">
+      <c r="E124" s="26"/>
+    </row>
+    <row r="125" spans="3:6">
+      <c r="C125" s="28"/>
+      <c r="D125" s="28"/>
+      <c r="E125" s="30"/>
+      <c r="F125" s="30"/>
+    </row>
+    <row r="126" spans="4:5">
+      <c r="D126" s="26" t="s">
         <v>179</v>
       </c>
-      <c r="E125" s="26"/>
-      <c r="F125" s="25" t="s">
+      <c r="E126" s="26"/>
+    </row>
+    <row r="127" spans="5:5">
+      <c r="E127" s="25" t="s">
         <v>180</v>
       </c>
-      <c r="G125" s="25" t="s">
+    </row>
+    <row r="128" spans="1:5">
+      <c r="A128" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B128" s="25" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="126" spans="5:5">
-      <c r="E126" s="33" t="s">
+      <c r="E128" s="25" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
-      <c r="A127" s="29" t="s">
+    <row r="129" spans="3:6">
+      <c r="C129" s="28"/>
+      <c r="D129" s="28"/>
+      <c r="E129" s="30"/>
+      <c r="F129" s="30"/>
+    </row>
+    <row r="130" spans="1:3">
+      <c r="A130" s="25" t="s">
         <v>183</v>
       </c>
-      <c r="E127" s="26"/>
-    </row>
-    <row r="128" spans="3:6">
-      <c r="C128" s="28"/>
-      <c r="D128" s="28"/>
-      <c r="E128" s="30"/>
-      <c r="F128" s="30"/>
-    </row>
-    <row r="129" spans="4:5">
-      <c r="D129" s="26" t="s">
+      <c r="C130" s="26" t="s">
         <v>184</v>
       </c>
-      <c r="E129" s="26"/>
-    </row>
-    <row r="130" spans="5:5">
-      <c r="E130" s="25" t="s">
+    </row>
+    <row r="131" spans="4:4">
+      <c r="D131" s="25" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="131" spans="1:5">
-      <c r="A131" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B131" s="25" t="s">
+    <row r="132" spans="4:4">
+      <c r="D132" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="E131" s="25" t="s">
+    </row>
+    <row r="133" spans="1:5">
+      <c r="A133" s="25" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="132" spans="3:6">
-      <c r="C132" s="28"/>
-      <c r="D132" s="28"/>
-      <c r="E132" s="30"/>
-      <c r="F132" s="30"/>
-    </row>
-    <row r="133" spans="1:3">
-      <c r="A133" s="25" t="s">
+      <c r="D133" s="25"/>
+      <c r="E133" s="25" t="s">
         <v>188</v>
-      </c>
-      <c r="C133" s="26" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="134" spans="4:4">
       <c r="D134" s="25" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6">
+      <c r="A135" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B135" s="25" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="135" spans="4:4">
       <c r="D135" s="25" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="136" spans="1:5">
-      <c r="A136" s="25" t="s">
+      <c r="F135" s="30" t="s">
         <v>192</v>
       </c>
-      <c r="D136" s="25"/>
-      <c r="E136" s="25" t="s">
+    </row>
+    <row r="137" spans="4:5">
+      <c r="D137" s="26" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="137" spans="4:4">
-      <c r="D137" s="25" t="s">
+      <c r="E137" s="26"/>
+    </row>
+    <row r="138" spans="5:5">
+      <c r="E138" s="26" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="138" spans="1:6">
-      <c r="A138" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="B138" s="25" t="s">
+    <row r="139" spans="5:5">
+      <c r="E139" s="26" t="s">
         <v>195</v>
       </c>
-      <c r="D138" s="25" t="s">
+    </row>
+    <row r="140" spans="1:5">
+      <c r="A140" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B140" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="F138" s="30" t="s">
+      <c r="E140" s="26" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="140" spans="4:5">
-      <c r="D140" s="26" t="s">
+    <row r="141" ht="13" customHeight="1" spans="2:5">
+      <c r="B141" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="E140" s="26"/>
-    </row>
-    <row r="141" spans="5:5">
-      <c r="E141" s="26" t="s">
+      <c r="E141" s="26"/>
+    </row>
+    <row r="142" ht="13" customHeight="1" spans="2:5">
+      <c r="B142" s="29" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="142" spans="5:5">
-      <c r="E142" s="26" t="s">
+      <c r="E142" s="26"/>
+    </row>
+    <row r="143" ht="13" customHeight="1" spans="1:5">
+      <c r="A143" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B143" s="29" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="143" spans="1:5">
-      <c r="A143" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="B143" s="25" t="s">
+      <c r="E143" s="26"/>
+    </row>
+    <row r="144" ht="13" customHeight="1" spans="2:5">
+      <c r="B144" s="29"/>
+      <c r="E144" s="26" t="s">
         <v>201</v>
       </c>
-      <c r="E143" s="26" t="s">
+    </row>
+    <row r="145" ht="13" customHeight="1" spans="1:5">
+      <c r="A145" s="25" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="144" ht="13" customHeight="1" spans="2:5">
-      <c r="B144" s="25" t="s">
+      <c r="B145" s="29" t="s">
         <v>203</v>
       </c>
-      <c r="E144" s="26"/>
-    </row>
-    <row r="145" ht="13" customHeight="1" spans="2:5">
-      <c r="B145" s="29" t="s">
+      <c r="E145" s="26"/>
+    </row>
+    <row r="146" ht="13" customHeight="1" spans="2:5">
+      <c r="B146" s="29"/>
+      <c r="E146" s="26"/>
+    </row>
+    <row r="147" ht="13" customHeight="1" spans="1:5">
+      <c r="A147" s="25" t="s">
         <v>204</v>
       </c>
-      <c r="E145" s="26"/>
-    </row>
-    <row r="146" ht="13" customHeight="1" spans="1:5">
-      <c r="A146" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B146" s="29" t="s">
+      <c r="E147" s="26" t="s">
         <v>205</v>
       </c>
-      <c r="E146" s="26"/>
-    </row>
-    <row r="147" ht="13" customHeight="1" spans="2:5">
-      <c r="B147" s="29"/>
-      <c r="E147" s="26" t="s">
+    </row>
+    <row r="148" ht="29" spans="1:8">
+      <c r="A148" s="25" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="148" ht="13" customHeight="1" spans="1:5">
-      <c r="A148" s="25" t="s">
+      <c r="B148" s="29"/>
+      <c r="E148" s="26"/>
+      <c r="H148" s="34" t="s">
         <v>207</v>
       </c>
-      <c r="B148" s="29" t="s">
+    </row>
+    <row r="149" ht="13" customHeight="1" spans="1:5">
+      <c r="A149" s="25" t="s">
         <v>208</v>
       </c>
-      <c r="E148" s="26"/>
-    </row>
-    <row r="149" ht="13" customHeight="1" spans="2:5">
       <c r="B149" s="29"/>
       <c r="E149" s="26"/>
     </row>
-    <row r="150" ht="13" customHeight="1" spans="1:7">
+    <row r="150" ht="13" customHeight="1" spans="1:8">
       <c r="A150" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="E150" s="26" t="s">
+      <c r="B150" s="29"/>
+      <c r="E150" s="26"/>
+      <c r="H150" s="28" t="s">
         <v>210</v>
       </c>
-      <c r="G150" s="34" t="s">
+    </row>
+    <row r="151" ht="13" customHeight="1" spans="1:6">
+      <c r="A151" s="25" t="s">
         <v>211</v>
-      </c>
-    </row>
-    <row r="151" ht="13" customHeight="1" spans="1:7">
-      <c r="A151" s="25" t="s">
-        <v>212</v>
       </c>
       <c r="B151" s="29"/>
       <c r="E151" s="26"/>
-      <c r="G151" s="25" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="152" ht="13" customHeight="1" spans="1:5">
-      <c r="A152" s="25" t="s">
-        <v>214</v>
-      </c>
+      <c r="F151" s="25" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="152" ht="13" customHeight="1" spans="2:8">
       <c r="B152" s="29"/>
       <c r="E152" s="26"/>
-    </row>
-    <row r="153" ht="13" customHeight="1" spans="1:7">
-      <c r="A153" s="25" t="s">
-        <v>215</v>
-      </c>
+      <c r="F152" s="25" t="s">
+        <v>213</v>
+      </c>
+      <c r="H152" s="25" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="153" ht="13" customHeight="1" spans="2:8">
       <c r="B153" s="29"/>
       <c r="E153" s="26"/>
-      <c r="G153" s="28" t="s">
+      <c r="F153" s="25" t="s">
+        <v>215</v>
+      </c>
+      <c r="H153" s="25" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="154" ht="13" customHeight="1" spans="1:6">
-      <c r="A154" s="25" t="s">
+    <row r="154" ht="13" customHeight="1" spans="2:8">
+      <c r="B154" s="29"/>
+      <c r="E154" s="26" t="s">
         <v>217</v>
       </c>
-      <c r="B154" s="29"/>
-      <c r="E154" s="26"/>
-      <c r="F154" s="25" t="s">
+      <c r="H154" s="25" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="155" ht="13" customHeight="1" spans="2:7">
+    <row r="155" ht="13" customHeight="1" spans="2:6">
       <c r="B155" s="29"/>
       <c r="E155" s="26"/>
       <c r="F155" s="25" t="s">
         <v>219</v>
       </c>
-      <c r="G155" s="25" t="s">
+    </row>
+    <row r="156" ht="13" customHeight="1" spans="1:8">
+      <c r="A156" s="25" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="156" ht="13" customHeight="1" spans="2:7">
       <c r="B156" s="29"/>
       <c r="E156" s="26"/>
-      <c r="F156" s="25" t="s">
+      <c r="H156" s="25" t="s">
         <v>221</v>
       </c>
-      <c r="G156" s="25" t="s">
+    </row>
+    <row r="157" ht="13" customHeight="1" spans="2:6">
+      <c r="B157" s="29"/>
+      <c r="E157" s="26"/>
+      <c r="F157" s="25" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="157" ht="13" customHeight="1" spans="2:7">
-      <c r="B157" s="29"/>
-      <c r="E157" s="26" t="s">
-        <v>223</v>
-      </c>
-      <c r="G157" s="25" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="158" ht="13" customHeight="1" spans="2:6">
+    <row r="158" ht="13" customHeight="1" spans="1:6">
+      <c r="A158" s="25" t="s">
+        <v>211</v>
+      </c>
       <c r="B158" s="29"/>
       <c r="E158" s="26"/>
       <c r="F158" s="25" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="159" ht="13" customHeight="1" spans="1:7">
-      <c r="A159" s="25" t="s">
-        <v>226</v>
-      </c>
+        <v>223</v>
+      </c>
+    </row>
+    <row r="159" spans="2:5">
       <c r="B159" s="29"/>
       <c r="E159" s="26"/>
-      <c r="G159" s="25" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="160" ht="13" customHeight="1" spans="2:6">
+    </row>
+    <row r="160" spans="2:5">
       <c r="B160" s="29"/>
-      <c r="E160" s="26"/>
-      <c r="F160" s="25" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="161" ht="13" customHeight="1" spans="1:6">
+      <c r="E160" s="26" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6">
       <c r="A161" s="25" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B161" s="29"/>
       <c r="E161" s="26"/>
-      <c r="F161" s="25" t="s">
-        <v>229</v>
+      <c r="F161" s="30" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="162" spans="2:5">
-      <c r="B162" s="29"/>
+      <c r="B162" s="35" t="s">
+        <v>226</v>
+      </c>
       <c r="E162" s="26"/>
     </row>
     <row r="163" spans="2:5">
       <c r="B163" s="29"/>
-      <c r="E163" s="26" t="s">
+      <c r="E163" s="26"/>
+    </row>
+    <row r="164" spans="4:5">
+      <c r="D164" s="26" t="s">
+        <v>227</v>
+      </c>
+      <c r="E164" s="26"/>
+    </row>
+    <row r="165" spans="5:5">
+      <c r="E165" s="25" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="166" spans="4:5">
+      <c r="D166" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="E166" s="26"/>
+    </row>
+    <row r="167" spans="5:5">
+      <c r="E167" s="25" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="164" spans="1:6">
-      <c r="A164" s="25" t="s">
-        <v>226</v>
-      </c>
-      <c r="B164" s="29"/>
-      <c r="E164" s="26"/>
-      <c r="F164" s="30" t="s">
+    <row r="168" spans="1:5">
+      <c r="A168" s="25" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="165" spans="2:5">
-      <c r="B165" s="35" t="s">
+      <c r="E168" s="25" t="s">
         <v>232</v>
-      </c>
-      <c r="E165" s="26"/>
-    </row>
-    <row r="166" spans="2:5">
-      <c r="B166" s="29"/>
-      <c r="E166" s="26"/>
-    </row>
-    <row r="167" spans="4:5">
-      <c r="D167" s="26" t="s">
-        <v>233</v>
-      </c>
-      <c r="E167" s="26"/>
-    </row>
-    <row r="168" spans="5:5">
-      <c r="E168" s="25" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="169" spans="4:5">
-      <c r="D169" s="26" t="s">
-        <v>235</v>
-      </c>
-      <c r="E169" s="26"/>
-    </row>
-    <row r="170" spans="5:5">
-      <c r="E170" s="25" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="171" spans="1:5">
-      <c r="A171" s="25" t="s">
-        <v>237</v>
-      </c>
-      <c r="E171" s="25" t="s">
-        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -3885,7 +3851,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="13" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3899,18 +3865,18 @@
         <v>17</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>18</v>
+        <v>234</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>19</v>
+        <v>235</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>20</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="3:6">
       <c r="C3" s="14" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D3" s="15"/>
       <c r="E3" s="15"/>
@@ -3919,7 +3885,7 @@
     <row r="4" spans="3:6">
       <c r="C4" s="14"/>
       <c r="D4" s="15" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="15"/>
@@ -3927,35 +3893,35 @@
     <row r="5" spans="3:6">
       <c r="C5" s="14"/>
       <c r="D5" s="15" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E5" s="15"/>
       <c r="F5" s="15"/>
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="13" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="15"/>
       <c r="E6" s="15" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="F6" s="15"/>
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="16" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="15"/>
       <c r="F7" s="15" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8" spans="2:6">
       <c r="B8" s="17" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="15"/>
@@ -3966,7 +3932,7 @@
       <c r="C9" s="14"/>
       <c r="D9" s="15"/>
       <c r="E9" s="13" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F9" s="15"/>
     </row>
@@ -3975,10 +3941,10 @@
       <c r="C10" s="14"/>
       <c r="D10" s="15"/>
       <c r="E10" s="13" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="11" spans="2:6">
@@ -3990,10 +3956,10 @@
     <row r="12" spans="3:6">
       <c r="C12" s="14"/>
       <c r="D12" s="15" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F12" s="15"/>
     </row>
@@ -4001,14 +3967,14 @@
       <c r="C13" s="14"/>
       <c r="D13" s="15"/>
       <c r="E13" s="15" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F13" s="15"/>
     </row>
     <row r="14" spans="3:6">
       <c r="C14" s="14"/>
       <c r="D14" s="15" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
@@ -4016,7 +3982,7 @@
     <row r="15" spans="3:6">
       <c r="C15" s="14"/>
       <c r="D15" s="15" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E15" s="15"/>
       <c r="F15" s="15"/>
@@ -4024,17 +3990,17 @@
     <row r="16" spans="3:6">
       <c r="C16" s="14"/>
       <c r="D16" s="15" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" spans="3:6">
       <c r="C17" s="14"/>
       <c r="D17" s="15"/>
       <c r="E17" s="15" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="F17" s="15"/>
     </row>
@@ -4046,29 +4012,29 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="13" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="15" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E19" s="15"/>
       <c r="F19" s="15"/>
     </row>
     <row r="20" spans="2:6">
       <c r="B20" s="13" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C20" s="14"/>
       <c r="D20" s="15"/>
       <c r="E20" s="15" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F20" s="15"/>
     </row>
     <row r="21" spans="2:6">
       <c r="B21" s="13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C21" s="14"/>
       <c r="D21" s="15"/>
@@ -4079,7 +4045,7 @@
       <c r="C22" s="14"/>
       <c r="D22" s="15"/>
       <c r="E22" s="15" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="F22" s="15"/>
     </row>
@@ -4097,7 +4063,7 @@
     </row>
     <row r="25" spans="3:6">
       <c r="C25" s="14" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
@@ -4106,7 +4072,7 @@
     <row r="26" spans="3:6">
       <c r="C26" s="14"/>
       <c r="D26" s="15" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E26" s="15"/>
       <c r="F26" s="15"/>
@@ -4114,7 +4080,7 @@
     <row r="27" spans="3:6">
       <c r="C27" s="14"/>
       <c r="D27" s="15" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="E27" s="15"/>
       <c r="F27" s="15"/>
@@ -4122,7 +4088,7 @@
     <row r="28" spans="3:6">
       <c r="C28" s="14"/>
       <c r="D28" s="15" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E28" s="15"/>
       <c r="F28" s="15"/>
@@ -4130,7 +4096,7 @@
     <row r="29" spans="3:6">
       <c r="C29" s="14"/>
       <c r="D29" s="15" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E29" s="15"/>
       <c r="F29" s="15"/>
@@ -4138,14 +4104,14 @@
     <row r="30" spans="3:6">
       <c r="C30" s="14"/>
       <c r="D30" s="15" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E30" s="15"/>
       <c r="F30" s="15"/>
     </row>
     <row r="31" spans="3:6">
       <c r="C31" s="14" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="15"/>
@@ -4154,7 +4120,7 @@
     <row r="32" spans="3:6">
       <c r="C32" s="14"/>
       <c r="D32" s="15" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E32" s="15"/>
       <c r="F32" s="15"/>
@@ -4162,7 +4128,7 @@
     <row r="33" spans="3:6">
       <c r="C33" s="14"/>
       <c r="D33" s="15" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="E33" s="15"/>
       <c r="F33" s="15"/>
@@ -4175,7 +4141,7 @@
     <row r="35" spans="3:5">
       <c r="C35" s="14"/>
       <c r="D35" s="15" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E35" s="15"/>
     </row>
@@ -4183,7 +4149,7 @@
       <c r="C36" s="14"/>
       <c r="D36" s="15"/>
       <c r="E36" s="15" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="37" spans="3:5">
@@ -4194,18 +4160,18 @@
     <row r="38" spans="3:5">
       <c r="C38" s="14"/>
       <c r="D38" s="15" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="E38" s="15"/>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="13" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C39" s="14"/>
       <c r="D39" s="15"/>
       <c r="E39" s="15" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="40" spans="3:5">
@@ -4218,18 +4184,18 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="13" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C42" s="14"/>
       <c r="D42" s="13" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:8">
       <c r="A43" s="18"/>
       <c r="B43" s="18"/>
       <c r="C43" s="19" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D43" s="18"/>
       <c r="E43" s="18"/>
@@ -4239,14 +4205,14 @@
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:8">
       <c r="A44" s="18" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C44" s="19"/>
       <c r="D44" s="18" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="E44" s="18"/>
       <c r="F44" s="18"/>
@@ -4255,14 +4221,14 @@
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:8">
       <c r="A45" s="13" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C45" s="19"/>
       <c r="D45" s="18" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="E45" s="18"/>
       <c r="F45" s="18"/>
@@ -4272,11 +4238,11 @@
     <row r="46" ht="16" customHeight="1" spans="1:8">
       <c r="A46" s="18"/>
       <c r="B46" s="18" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C46" s="19"/>
       <c r="D46" s="18" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="E46" s="18"/>
       <c r="F46" s="18"/>
@@ -4286,11 +4252,11 @@
     <row r="47" ht="16" customHeight="1" spans="1:8">
       <c r="A47" s="18"/>
       <c r="B47" s="18" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C47" s="19"/>
       <c r="D47" s="18" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E47" s="18"/>
       <c r="F47" s="18"/>
@@ -4300,11 +4266,11 @@
     <row r="48" ht="16" customHeight="1" spans="1:8">
       <c r="A48" s="18"/>
       <c r="B48" s="18" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C48" s="19"/>
       <c r="D48" s="18" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E48" s="18"/>
       <c r="F48" s="18"/>
@@ -4324,7 +4290,7 @@
       <c r="B50" s="18"/>
       <c r="C50" s="19"/>
       <c r="D50" s="15" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="E50" s="18"/>
       <c r="F50" s="18"/>
@@ -4335,7 +4301,7 @@
       <c r="B51" s="18"/>
       <c r="C51" s="19"/>
       <c r="D51" s="15" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="E51" s="18"/>
       <c r="F51" s="18"/>
@@ -4343,13 +4309,13 @@
     </row>
     <row r="52" ht="16" customHeight="1" spans="1:8">
       <c r="A52" s="18" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B52" s="18"/>
       <c r="C52" s="19"/>
       <c r="D52" s="15"/>
       <c r="E52" s="18" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F52" s="18"/>
       <c r="H52" s="20"/>
@@ -4357,12 +4323,12 @@
     <row r="53" ht="74" customHeight="1" spans="1:8">
       <c r="A53" s="18"/>
       <c r="B53" s="21" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C53" s="19"/>
       <c r="D53" s="15"/>
       <c r="E53" s="21" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="F53" s="18"/>
       <c r="H53" s="20"/>
@@ -4373,7 +4339,7 @@
       <c r="C54" s="19"/>
       <c r="D54" s="15"/>
       <c r="E54" s="21" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F54" s="18"/>
       <c r="H54" s="20"/>
@@ -4381,26 +4347,26 @@
     <row r="55" ht="29" customHeight="1" spans="1:8">
       <c r="A55" s="18"/>
       <c r="B55" s="21" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C55" s="19"/>
       <c r="D55" s="15"/>
       <c r="E55" s="21" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="F55" s="18"/>
       <c r="H55" s="20"/>
     </row>
     <row r="56" ht="16" customHeight="1" spans="1:8">
       <c r="A56" s="18" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="B56" s="18" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C56" s="19"/>
       <c r="D56" s="18" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="E56" s="18"/>
       <c r="F56" s="18"/>
@@ -4412,7 +4378,7 @@
       <c r="C57" s="19"/>
       <c r="D57" s="18"/>
       <c r="E57" s="18" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="F57" s="18"/>
       <c r="H57" s="20"/>
@@ -4423,7 +4389,7 @@
       <c r="C58" s="19"/>
       <c r="D58" s="18"/>
       <c r="E58" s="18" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="F58" s="18"/>
       <c r="H58" s="20"/>
@@ -4434,7 +4400,7 @@
       <c r="C59" s="19"/>
       <c r="D59" s="18"/>
       <c r="E59" s="18" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="F59" s="18"/>
       <c r="H59" s="20"/>
@@ -4445,7 +4411,7 @@
       <c r="C60" s="19"/>
       <c r="D60" s="18"/>
       <c r="E60" s="18" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="F60" s="18"/>
       <c r="H60" s="20"/>
@@ -4456,7 +4422,7 @@
       <c r="C61" s="19"/>
       <c r="D61" s="18"/>
       <c r="E61" s="18" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F61" s="18"/>
       <c r="H61" s="20"/>
@@ -4464,11 +4430,11 @@
     <row r="62" ht="16" customHeight="1" spans="1:8">
       <c r="A62" s="18"/>
       <c r="B62" s="18" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C62" s="19"/>
       <c r="D62" s="18" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E62" s="18"/>
       <c r="F62" s="18"/>
@@ -4477,11 +4443,11 @@
     <row r="63" ht="16" customHeight="1" spans="1:8">
       <c r="A63" s="18"/>
       <c r="B63" s="18" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C63" s="19"/>
       <c r="D63" s="18" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="E63" s="18"/>
       <c r="F63" s="18"/>
@@ -4490,11 +4456,11 @@
     <row r="64" ht="16" customHeight="1" spans="1:8">
       <c r="A64" s="18"/>
       <c r="B64" s="18" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C64" s="19"/>
       <c r="D64" s="18" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E64" s="18"/>
       <c r="F64" s="18"/>
@@ -4503,11 +4469,11 @@
     <row r="65" ht="16" customHeight="1" spans="1:8">
       <c r="A65" s="18"/>
       <c r="B65" s="18" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="18" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E65" s="18"/>
       <c r="F65" s="18"/>
@@ -4515,13 +4481,13 @@
     </row>
     <row r="66" ht="16" customHeight="1" spans="1:8">
       <c r="A66" s="18" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B66" s="18"/>
       <c r="C66" s="19"/>
       <c r="D66" s="18"/>
       <c r="E66" s="18" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="F66" s="18"/>
       <c r="H66" s="20"/>
@@ -4532,19 +4498,19 @@
       <c r="D67" s="18"/>
       <c r="E67" s="18"/>
       <c r="F67" s="18" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="H67" s="20"/>
     </row>
     <row r="68" ht="43" customHeight="1" spans="1:8">
       <c r="A68" s="18"/>
       <c r="B68" s="21" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C68" s="19"/>
       <c r="D68" s="18"/>
       <c r="E68" s="18" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="F68" s="18"/>
       <c r="H68" s="20"/>
@@ -4552,12 +4518,12 @@
     <row r="69" ht="14" customHeight="1" spans="1:8">
       <c r="A69" s="18"/>
       <c r="B69" s="22" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C69" s="19"/>
       <c r="D69" s="18"/>
       <c r="E69" s="18" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="F69" s="18"/>
       <c r="H69" s="20"/>
@@ -4565,12 +4531,12 @@
     <row r="70" ht="16" customHeight="1" spans="1:8">
       <c r="A70" s="18"/>
       <c r="B70" s="18" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C70" s="19"/>
       <c r="D70" s="18"/>
       <c r="E70" s="18" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="F70" s="18"/>
       <c r="H70" s="20"/>
@@ -4578,12 +4544,12 @@
     <row r="71" ht="16" customHeight="1" spans="1:8">
       <c r="A71" s="18"/>
       <c r="B71" s="18" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="C71" s="19"/>
       <c r="D71" s="18"/>
       <c r="E71" s="18" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="F71" s="18"/>
       <c r="H71" s="20"/>
@@ -4592,7 +4558,7 @@
       <c r="A72" s="18"/>
       <c r="B72" s="18"/>
       <c r="C72" s="19" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D72" s="18"/>
       <c r="E72" s="18"/>
@@ -4603,7 +4569,7 @@
       <c r="B73" s="18"/>
       <c r="C73" s="19"/>
       <c r="D73" s="18" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="E73" s="18"/>
       <c r="F73" s="18"/>
@@ -4614,7 +4580,7 @@
       <c r="C74" s="19"/>
       <c r="D74" s="18"/>
       <c r="E74" s="18" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="F74" s="18"/>
     </row>
@@ -4623,7 +4589,7 @@
       <c r="B75" s="18"/>
       <c r="C75" s="19"/>
       <c r="D75" s="18" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="E75" s="18"/>
       <c r="F75" s="18"/>
@@ -4634,7 +4600,7 @@
       <c r="C76" s="19"/>
       <c r="D76" s="18"/>
       <c r="E76" s="18" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F76" s="18"/>
     </row>
@@ -4643,7 +4609,7 @@
       <c r="B77" s="18"/>
       <c r="C77" s="19"/>
       <c r="D77" s="18" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="E77" s="18"/>
       <c r="F77" s="18"/>
@@ -4654,7 +4620,7 @@
       <c r="C78" s="19"/>
       <c r="D78" s="18"/>
       <c r="E78" s="18" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F78" s="18"/>
     </row>
@@ -4664,7 +4630,7 @@
       <c r="C79" s="19"/>
       <c r="D79" s="18"/>
       <c r="E79" s="18" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="F79" s="18"/>
     </row>
@@ -4672,7 +4638,7 @@
       <c r="A80" s="18"/>
       <c r="B80" s="18"/>
       <c r="C80" s="19" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D80" s="18"/>
       <c r="E80" s="18"/>
@@ -4683,7 +4649,7 @@
       <c r="B81" s="21"/>
       <c r="C81" s="23"/>
       <c r="D81" s="18" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E81" s="18"/>
       <c r="F81" s="21"/>
@@ -4693,7 +4659,7 @@
       <c r="B82" s="18"/>
       <c r="C82" s="19"/>
       <c r="D82" s="18" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="E82" s="18"/>
       <c r="F82" s="18"/>
@@ -4703,7 +4669,7 @@
       <c r="B83" s="18"/>
       <c r="C83" s="19"/>
       <c r="D83" s="18" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E83" s="18"/>
       <c r="F83" s="18"/>
@@ -4711,7 +4677,7 @@
     <row r="84" spans="1:6">
       <c r="A84" s="18"/>
       <c r="B84" s="18" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="C84" s="19"/>
       <c r="D84" s="18"/>
@@ -4720,13 +4686,13 @@
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="18" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="B85" s="18"/>
       <c r="C85" s="19"/>
       <c r="D85" s="18"/>
       <c r="E85" s="18" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="F85" s="18"/>
     </row>
@@ -4743,7 +4709,7 @@
       <c r="B87" s="18"/>
       <c r="C87" s="19"/>
       <c r="D87" s="18" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E87" s="18"/>
       <c r="F87" s="18"/>
@@ -4754,7 +4720,7 @@
       <c r="C88" s="19"/>
       <c r="D88" s="18"/>
       <c r="E88" s="18" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="F88" s="18"/>
     </row>
@@ -4764,7 +4730,7 @@
       <c r="C89" s="19"/>
       <c r="D89" s="18"/>
       <c r="E89" s="18" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="F89" s="18"/>
     </row>
@@ -4773,7 +4739,7 @@
       <c r="B90" s="18"/>
       <c r="C90" s="19"/>
       <c r="D90" s="18" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="E90" s="18"/>
       <c r="F90" s="18"/>
@@ -4783,7 +4749,7 @@
       <c r="B91" s="18"/>
       <c r="C91" s="19"/>
       <c r="D91" s="18" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="E91" s="18"/>
       <c r="F91" s="18"/>
@@ -4824,7 +4790,7 @@
   <sheetData>
     <row r="1" ht="14" customHeight="1" spans="2:2">
       <c r="B1" s="6" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:8">
@@ -4838,103 +4804,103 @@
         <v>17</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>18</v>
+        <v>234</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>19</v>
+        <v>235</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>20</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" customHeight="1" spans="2:7">
       <c r="B3" s="6" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="G3" s="7"/>
     </row>
     <row r="4" customHeight="1" spans="3:7">
       <c r="C4" s="8" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="G4" s="7"/>
     </row>
     <row r="5" customHeight="1" spans="3:7">
       <c r="C5" s="9" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="G5" s="7"/>
     </row>
     <row r="6" customHeight="1" spans="3:7">
       <c r="C6" s="9" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="G6" s="7"/>
     </row>
     <row r="7" customHeight="1" spans="2:3">
       <c r="B7" s="6" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8" customHeight="1" spans="2:3">
       <c r="B8" s="6" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="9" customHeight="1" spans="2:3">
       <c r="B9" s="6" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
     </row>
     <row r="10" customHeight="1" spans="3:3">
       <c r="C10" s="9" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="11" customHeight="1" spans="3:3">
       <c r="C11" s="9" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="12" customHeight="1" spans="1:3">
       <c r="A12" s="6" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
     </row>
     <row r="13" customHeight="1" spans="2:3">
       <c r="B13" s="6" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
     </row>
     <row r="14" customHeight="1" spans="3:3">
       <c r="C14" s="9" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
     </row>
     <row r="15" customHeight="1" spans="3:3">
       <c r="C15" s="9" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="5:5">
@@ -4942,23 +4908,23 @@
     </row>
     <row r="19" customHeight="1" spans="2:3">
       <c r="B19" s="6" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="21" customHeight="1" spans="1:3">
       <c r="A21" s="6" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="22" customHeight="1" spans="4:4">
       <c r="D22" s="10" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="26" customHeight="1" spans="2:2">
@@ -5053,44 +5019,44 @@
         <v>17</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>18</v>
+        <v>234</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>19</v>
+        <v>235</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>20</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="4" spans="3:3">
       <c r="C4" s="4" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="4" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="6" spans="4:4">
       <c r="D6" s="4" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
     </row>
     <row r="7" spans="4:4">
       <c r="D7" s="4" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -5127,28 +5093,28 @@
         <v>17</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>18</v>
+        <v>234</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>19</v>
+        <v>235</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>20</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="3:3">
       <c r="C3" s="1" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="4" spans="4:4">
       <c r="D4" s="3" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="5" spans="4:4">
       <c r="D5" s="3" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HC PROFILE UPDATE AND py adv git update
</commit_message>
<xml_diff>
--- a/p/py-25/py-libs/pandas/topic-list_pandas.xlsx
+++ b/p/py-25/py-libs/pandas/topic-list_pandas.xlsx
@@ -1382,7 +1382,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="40">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1469,13 +1469,6 @@
     <font>
       <sz val="10.5"/>
       <color rgb="FF080808"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -1637,12 +1630,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF00622F"/>
-      <name val="Bahnschrift"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="10.5"/>
       <color rgb="FF00622F"/>
       <name val="Consolas"/>
@@ -1658,6 +1645,12 @@
       <sz val="10.5"/>
       <color rgb="FF00622F"/>
       <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00622F"/>
+      <name val="Bahnschrift"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -1994,148 +1987,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2208,12 +2201,12 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>